<commit_message>
feat(excel): add VaR/CVaR to Performance tab and metric descriptions
Performance tab:
- Populate var_95 and cvar_95 in every perf row (portfolio, holdings,
  benchmarks) via _populate_perf_row, using the existing compute_var
  and compute_cvar helpers.
- Add two new columns 'VaR 95%' and 'CVaR 95%' to the Performance
  table, placed right after Max DD in the risk group.
- Widen the merged note cell to the new last column.

Legend:
- Add a 'Description' column with investor-friendly explanations for
  CAGR, Alpha, Beta, Max DD, Volatility, Sharpe, Sortino, VaR, CVaR.
  Each description follows the same pattern: what it measures, how to
  read it, and concrete numeric anchors.
- Widen column B to 80 chars, enable wrap_text, bump row height to 48
  for readability.

Regenerate output/sample/portfolio_dashboard_sample.xlsx to reflect
the new columns and legend.
</commit_message>
<xml_diff>
--- a/output/sample/portfolio_dashboard_sample.xlsx
+++ b/output/sample/portfolio_dashboard_sample.xlsx
@@ -254,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -382,6 +382,12 @@
     </xf>
     <xf numFmtId="2" fontId="23" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -811,7 +817,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>80934.80267948778</v>
+        <v>80948.91581741307</v>
       </c>
       <c r="D5" s="2" t="n"/>
     </row>
@@ -822,7 +828,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>26794.80267948778</v>
+        <v>26808.91581741307</v>
       </c>
       <c r="D6" s="2" t="n"/>
     </row>
@@ -833,7 +839,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>49.49169316492017</v>
+        <v>49.5177610221889</v>
       </c>
       <c r="D7" s="2" t="n"/>
     </row>
@@ -897,7 +903,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>64.77801723311731</v>
+        <v>64.78415805286481</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>65</v>
@@ -909,7 +915,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>41.75790478337835</v>
+        <v>41.77116920492907</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>55</v>
@@ -922,7 +928,7 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>20.58336679884454</v>
+        <v>20.57977816653656</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>25</v>
@@ -934,7 +940,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>24.1498199211525</v>
+        <v>24.14476795526446</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>8</v>
@@ -947,7 +953,7 @@
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>8.460803908866717</v>
+        <v>8.459328799641117</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>5</v>
@@ -959,7 +965,7 @@
         </is>
       </c>
       <c r="F14" s="22" t="n">
-        <v>15.53026313713126</v>
+        <v>15.5217931241751</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>11</v>
@@ -972,7 +978,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>6.177812059171433</v>
+        <v>6.176734980957511</v>
       </c>
       <c r="C15" s="18" t="n">
         <v>5</v>
@@ -984,7 +990,7 @@
         </is>
       </c>
       <c r="F15" s="17" t="n">
-        <v>10.66366665568281</v>
+        <v>10.66269639765878</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>14</v>
@@ -998,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="22" t="n">
-        <v>7.898345502655069</v>
+        <v>7.899573317972592</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>12</v>
@@ -1054,10 +1060,10 @@
         </is>
       </c>
       <c r="B21" s="28" t="n">
-        <v>12433.59985351562</v>
+        <v>12441.60034179688</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>15.3624886227922</v>
+        <v>15.36969361005393</v>
       </c>
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="12" t="inlineStr">
@@ -1076,7 +1082,7 @@
         <v>11547.61339873075</v>
       </c>
       <c r="C22" s="33" t="n">
-        <v>14.26779706186569</v>
+        <v>14.26530952530278</v>
       </c>
       <c r="D22" s="30" t="n"/>
       <c r="E22" s="34" t="inlineStr">
@@ -1095,7 +1101,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="C23" s="29" t="n">
-        <v>13.23905143133624</v>
+        <v>13.23674325269094</v>
       </c>
       <c r="D23" s="30" t="n"/>
       <c r="E23" s="35" t="inlineStr">
@@ -1111,10 +1117,10 @@
         </is>
       </c>
       <c r="B24" s="32" t="n">
-        <v>9963.177533948419</v>
+        <v>9967.849677611011</v>
       </c>
       <c r="C24" s="33" t="n">
-        <v>12.31012766337849</v>
+        <v>12.31375315772519</v>
       </c>
       <c r="D24" s="30" t="n"/>
       <c r="E24" s="34" t="inlineStr">
@@ -1130,10 +1136,10 @@
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>6883.919906616211</v>
+        <v>6880.860214233398</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>8.505512682692782</v>
+        <v>8.500249996866843</v>
       </c>
       <c r="D25" s="30" t="n"/>
       <c r="E25" s="12" t="inlineStr">
@@ -1148,7 +1154,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 09:47 v2.0</t>
+          <t>Generated 2026-05-04 10:02 v2.0</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1339,7 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 09:47 v2.0</t>
+          <t>Generated 2026-05-04 10:02 v2.0</t>
         </is>
       </c>
     </row>
@@ -1534,25 +1540,25 @@
         <v>128</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>155.4199981689453</v>
+        <v>155.5200042724609</v>
       </c>
       <c r="J4" s="28" t="n">
         <v>10240</v>
       </c>
       <c r="K4" s="28" t="n">
-        <v>12433.59985351562</v>
+        <v>12441.60034179688</v>
       </c>
       <c r="L4" s="29" t="n">
-        <v>15.3624886227922</v>
+        <v>15.36969361005393</v>
       </c>
       <c r="M4" s="29" t="n">
-        <v>23.71558945298844</v>
+        <v>23.72446300453892</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>2193.599853515625</v>
+        <v>2201.600341796875</v>
       </c>
       <c r="O4" s="29" t="n">
-        <v>21.42187356948853</v>
+        <v>21.50000333786011</v>
       </c>
       <c r="P4" s="27" t="inlineStr">
         <is>
@@ -1571,7 +1577,7 @@
       </c>
       <c r="S4" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -1622,10 +1628,10 @@
         <v>11547.61339873075</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>14.26779706186569</v>
+        <v>14.26530952530278</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>22.02567733822422</v>
+        <v>22.01974981856225</v>
       </c>
       <c r="N5" s="32" t="n">
         <v>9307.613398730755</v>
@@ -1650,7 +1656,7 @@
       </c>
       <c r="S5" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -1692,25 +1698,25 @@
         <v>570</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>664.2118355965613</v>
+        <v>664.5233118407341</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>8550</v>
       </c>
       <c r="K6" s="28" t="n">
-        <v>9963.177533948419</v>
+        <v>9967.849677611011</v>
       </c>
       <c r="L6" s="29" t="n">
-        <v>12.31012766337849</v>
+        <v>12.31375315772519</v>
       </c>
       <c r="M6" s="29" t="n">
-        <v>19.0035573627978</v>
+        <v>19.00735230313095</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>1413.177533948419</v>
+        <v>1417.849677611011</v>
       </c>
       <c r="O6" s="29" t="n">
-        <v>16.52839220992303</v>
+        <v>16.58303716504107</v>
       </c>
       <c r="P6" s="27" t="inlineStr">
         <is>
@@ -1729,7 +1735,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -1771,25 +1777,25 @@
         <v>56</v>
       </c>
       <c r="I7" s="32" t="n">
-        <v>76.48799896240234</v>
+        <v>76.45400238037109</v>
       </c>
       <c r="J7" s="32" t="n">
         <v>5040</v>
       </c>
       <c r="K7" s="32" t="n">
-        <v>6883.919906616211</v>
+        <v>6880.860214233398</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>8.505512682692782</v>
+        <v>8.500249996866843</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>13.13024548448883</v>
+        <v>13.12087746811576</v>
       </c>
       <c r="N7" s="32" t="n">
-        <v>1843.919906616211</v>
+        <v>1840.860214233398</v>
       </c>
       <c r="O7" s="33" t="n">
-        <v>36.58571243286133</v>
+        <v>36.52500425066267</v>
       </c>
       <c r="P7" s="31" t="inlineStr">
         <is>
@@ -1808,7 +1814,7 @@
       </c>
       <c r="S7" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -1850,25 +1856,25 @@
         <v>98</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>118.004997253418</v>
+        <v>118.0950012207031</v>
       </c>
       <c r="J8" s="28" t="n">
         <v>4900</v>
       </c>
       <c r="K8" s="28" t="n">
-        <v>5900.249862670898</v>
+        <v>5904.750061035156</v>
       </c>
       <c r="L8" s="29" t="n">
-        <v>7.290126950746573</v>
+        <v>7.294415251161368</v>
       </c>
       <c r="M8" s="29" t="n">
-        <v>11.25401372584703</v>
+        <v>11.25956633596908</v>
       </c>
       <c r="N8" s="28" t="n">
-        <v>1000.249862670898</v>
+        <v>1004.750061035156</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>20.41326250348772</v>
+        <v>20.50510328643176</v>
       </c>
       <c r="P8" s="27" t="inlineStr">
         <is>
@@ -1887,7 +1893,7 @@
       </c>
       <c r="S8" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -1938,10 +1944,10 @@
         <v>5699.399871826172</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v>7.041964251641569</v>
+        <v>7.040736511754693</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v>10.8709166356537</v>
+        <v>10.86799106968304</v>
       </c>
       <c r="N9" s="32" t="n">
         <v>1739.399871826172</v>
@@ -1966,7 +1972,7 @@
       </c>
       <c r="S9" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2023,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="L10" s="29" t="n">
-        <v>13.23905143133624</v>
+        <v>13.23674325269094</v>
       </c>
       <c r="M10" s="29" t="n">
         <v>64.31917363528412</v>
@@ -2045,7 +2051,7 @@
       </c>
       <c r="S10" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2102,7 @@
         <v>5944.107150852142</v>
       </c>
       <c r="L11" s="33" t="n">
-        <v>7.344315367508301</v>
+        <v>7.343034913845621</v>
       </c>
       <c r="M11" s="33" t="n">
         <v>35.68082636471589</v>
@@ -2124,7 +2130,7 @@
       </c>
       <c r="S11" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:01</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2181,7 @@
         <v>5000</v>
       </c>
       <c r="L12" s="29" t="n">
-        <v>6.177812059171433</v>
+        <v>6.176734980957511</v>
       </c>
       <c r="M12" s="29" t="n">
         <v>100</v>
@@ -2203,7 +2209,7 @@
       </c>
       <c r="S12" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:02</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2260,7 @@
         <v>6847.734948739668</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v>8.460803908866717</v>
+        <v>8.459328799641117</v>
       </c>
       <c r="M13" s="33" t="n">
         <v>100</v>
@@ -2282,14 +2288,14 @@
       </c>
       <c r="S13" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 09:46</t>
+          <t>2026-05-04 10:02</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 09:47 v2.0</t>
+          <t>Generated 2026-05-04 10:02 v2.0</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2326,7 +2332,9 @@
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2426,15 +2434,25 @@
       </c>
       <c r="Q4" s="11" t="inlineStr">
         <is>
+          <t>VaR 95%</t>
+        </is>
+      </c>
+      <c r="R4" s="11" t="inlineStr">
+        <is>
+          <t>CVaR 95%</t>
+        </is>
+      </c>
+      <c r="S4" s="11" t="inlineStr">
+        <is>
           <t>α (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="R4" s="11" t="inlineStr">
+      <c r="T4" s="11" t="inlineStr">
         <is>
           <t>β (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="S4" s="11" t="inlineStr">
+      <c r="U4" s="11" t="inlineStr">
         <is>
           <t>Period Used</t>
         </is>
@@ -2452,31 +2470,31 @@
         </is>
       </c>
       <c r="C5" s="44" t="n">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="D5" s="44" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="E5" s="44" t="n">
-        <v>6.07</v>
+        <v>6.09</v>
       </c>
       <c r="F5" s="44" t="n">
-        <v>4.17</v>
+        <v>4.19</v>
       </c>
       <c r="G5" s="44" t="n">
-        <v>6.74</v>
+        <v>6.76</v>
       </c>
       <c r="H5" s="44" t="n">
-        <v>7.15</v>
+        <v>7.17</v>
       </c>
       <c r="I5" s="44" t="n">
-        <v>22.18</v>
+        <v>22.21</v>
       </c>
       <c r="J5" s="44" t="n">
-        <v>49.14</v>
+        <v>49.17</v>
       </c>
       <c r="K5" s="44" t="n">
-        <v>45.31</v>
+        <v>45.34</v>
       </c>
       <c r="L5" s="44" t="n">
         <v>7.95</v>
@@ -2493,13 +2511,19 @@
       <c r="P5" s="45" t="n">
         <v>-13.91</v>
       </c>
-      <c r="Q5" s="44" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="R5" s="44" t="n">
+      <c r="Q5" s="45" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="R5" s="45" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="S5" s="44" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="T5" s="44" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="43" t="inlineStr">
+      <c r="U5" s="43" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2558,13 +2582,19 @@
       <c r="P6" s="46" t="n">
         <v>-20.22</v>
       </c>
-      <c r="Q6" s="29" t="n">
+      <c r="Q6" s="46" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="R6" s="46" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="S6" s="29" t="n">
         <v>5.17</v>
       </c>
-      <c r="R6" s="29" t="n">
+      <c r="T6" s="29" t="n">
         <v>0.3</v>
       </c>
-      <c r="S6" s="27" t="inlineStr">
+      <c r="U6" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2582,34 +2612,34 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>6.6</v>
+        <v>6.61</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>4.43</v>
+        <v>4.44</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>6.35</v>
+        <v>6.36</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>6.48</v>
+        <v>6.49</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>23.64</v>
+        <v>23.65</v>
       </c>
       <c r="J7" s="33" t="n">
-        <v>56.11</v>
+        <v>56.12</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>58.68</v>
+        <v>58.7</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>9.82</v>
+        <v>9.83</v>
       </c>
       <c r="M7" s="33" t="n">
         <v>15.1</v>
@@ -2624,12 +2654,18 @@
         <v>-20.07</v>
       </c>
       <c r="Q7" s="47" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="R7" s="47" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="S7" s="47" t="n">
         <v>-0.5</v>
       </c>
-      <c r="R7" s="33" t="n">
+      <c r="T7" s="33" t="n">
         <v>0.78</v>
       </c>
-      <c r="S7" s="31" t="inlineStr">
+      <c r="U7" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2689,12 +2725,18 @@
         <v>-17.35</v>
       </c>
       <c r="Q8" s="46" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="R8" s="46" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="S8" s="46" t="n">
         <v>-1.39</v>
       </c>
-      <c r="R8" s="29" t="n">
+      <c r="T8" s="29" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="S8" s="27" t="inlineStr">
+      <c r="U8" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2754,12 +2796,18 @@
         <v>-24.81</v>
       </c>
       <c r="Q9" s="47" t="n">
+        <v>-1.93</v>
+      </c>
+      <c r="R9" s="47" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="S9" s="47" t="n">
         <v>-3.89</v>
       </c>
-      <c r="R9" s="33" t="n">
+      <c r="T9" s="33" t="n">
         <v>0.79</v>
       </c>
-      <c r="S9" s="31" t="inlineStr">
+      <c r="U9" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2777,31 +2825,31 @@
         </is>
       </c>
       <c r="C10" s="46" t="n">
-        <v>-0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>5.93</v>
+        <v>5.94</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>3.93</v>
+        <v>3.95</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>5.04</v>
+        <v>5.05</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>5.33</v>
+        <v>5.34</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>21.7</v>
+        <v>21.71</v>
       </c>
       <c r="J10" s="29" t="n">
-        <v>55.64</v>
+        <v>55.65</v>
       </c>
       <c r="K10" s="29" t="n">
-        <v>63.24</v>
+        <v>63.25</v>
       </c>
       <c r="L10" s="29" t="n">
         <v>10.46</v>
@@ -2819,12 +2867,18 @@
         <v>-20.63</v>
       </c>
       <c r="Q10" s="46" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="R10" s="46" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="S10" s="46" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="R10" s="29" t="n">
+      <c r="T10" s="29" t="n">
         <v>0.86</v>
       </c>
-      <c r="S10" s="27" t="inlineStr">
+      <c r="U10" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2883,13 +2937,19 @@
       <c r="P11" s="47" t="n">
         <v>-25.91</v>
       </c>
-      <c r="Q11" s="33" t="n">
+      <c r="Q11" s="47" t="n">
+        <v>-2.26</v>
+      </c>
+      <c r="R11" s="47" t="n">
+        <v>-3.15</v>
+      </c>
+      <c r="S11" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="R11" s="33" t="n">
+      <c r="T11" s="33" t="n">
         <v>1.06</v>
       </c>
-      <c r="S11" s="31" t="inlineStr">
+      <c r="U11" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -2949,12 +3009,18 @@
         <v>-22.45</v>
       </c>
       <c r="Q12" s="46" t="n">
+        <v>-1.79</v>
+      </c>
+      <c r="R12" s="46" t="n">
+        <v>-2.66</v>
+      </c>
+      <c r="S12" s="46" t="n">
         <v>-0.13</v>
       </c>
-      <c r="R12" s="29" t="n">
+      <c r="T12" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="S12" s="27" t="inlineStr">
+      <c r="U12" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3013,13 +3079,19 @@
       <c r="P13" s="47" t="n">
         <v>-31.38</v>
       </c>
-      <c r="Q13" s="33" t="n">
+      <c r="Q13" s="47" t="n">
+        <v>-2.45</v>
+      </c>
+      <c r="R13" s="47" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="S13" s="33" t="n">
         <v>1.59</v>
       </c>
-      <c r="R13" s="33" t="n">
+      <c r="T13" s="33" t="n">
         <v>1.23</v>
       </c>
-      <c r="S13" s="31" t="inlineStr">
+      <c r="U13" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3078,13 +3150,19 @@
       <c r="P14" s="46" t="n">
         <v>-23.17</v>
       </c>
-      <c r="Q14" s="29" t="n">
+      <c r="Q14" s="46" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="R14" s="46" t="n">
+        <v>-2.64</v>
+      </c>
+      <c r="S14" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="R14" s="29" t="n">
+      <c r="T14" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="S14" s="27" t="inlineStr">
+      <c r="U14" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3102,34 +3180,34 @@
         </is>
       </c>
       <c r="C15" s="33" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="D15" s="33" t="n">
-        <v>1.18</v>
+        <v>1.26</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>7.55</v>
+        <v>7.63</v>
       </c>
       <c r="F15" s="33" t="n">
-        <v>4.46</v>
+        <v>4.54</v>
       </c>
       <c r="G15" s="33" t="n">
-        <v>5.61</v>
+        <v>5.69</v>
       </c>
       <c r="H15" s="33" t="n">
-        <v>6.01</v>
+        <v>6.09</v>
       </c>
       <c r="I15" s="33" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="J15" s="33" t="n">
-        <v>62.99</v>
+        <v>63.11</v>
       </c>
       <c r="K15" s="33" t="n">
-        <v>75.48</v>
+        <v>75.62</v>
       </c>
       <c r="L15" s="33" t="n">
-        <v>12.21</v>
+        <v>12.23</v>
       </c>
       <c r="M15" s="33" t="n">
         <v>14.24</v>
@@ -3143,13 +3221,19 @@
       <c r="P15" s="47" t="n">
         <v>-21.73</v>
       </c>
-      <c r="Q15" s="33" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="R15" s="33" t="n">
+      <c r="Q15" s="47" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="R15" s="47" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="S15" s="33" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="T15" s="33" t="n">
         <v>0.22</v>
       </c>
-      <c r="S15" s="31" t="inlineStr">
+      <c r="U15" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3158,7 +3242,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares VII PLC - iShares Nikkei 225 ETF JPY Acc</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
@@ -3167,54 +3251,60 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.95</v>
+        <v>0.04</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>1.25</v>
+        <v>0.93</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>7.99</v>
+        <v>9.6</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>4.94</v>
+        <v>10.93</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>6.85</v>
+        <v>10.3</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>7.08</v>
+        <v>17.9</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>24.9</v>
+        <v>44.84</v>
       </c>
       <c r="J16" s="29" t="n">
-        <v>63.17</v>
+        <v>73.92</v>
       </c>
       <c r="K16" s="29" t="n">
-        <v>70.66</v>
+        <v>57.6</v>
       </c>
       <c r="L16" s="29" t="n">
-        <v>11.57</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="M16" s="29" t="n">
-        <v>13.81</v>
+        <v>18.27</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.55</v>
+        <v>0.3</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.7</v>
+        <v>0.46</v>
       </c>
       <c r="P16" s="46" t="n">
-        <v>-21.07</v>
-      </c>
-      <c r="Q16" s="29" t="n">
-        <v>5.97</v>
-      </c>
-      <c r="R16" s="29" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="S16" s="27" t="inlineStr">
+        <v>-21.24</v>
+      </c>
+      <c r="Q16" s="46" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="R16" s="46" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="S16" s="29" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="T16" s="29" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="U16" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3223,7 +3313,7 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="B17" s="31" t="inlineStr">
@@ -3232,54 +3322,60 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>2.26</v>
+        <v>1.01</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>1.84</v>
+        <v>1.32</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>13.08</v>
+        <v>8.06</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>9.359999999999999</v>
+        <v>5.01</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>17.01</v>
+        <v>6.92</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>16.61</v>
+        <v>7.15</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>41.31</v>
+        <v>24.98</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>69.36</v>
+        <v>63.28</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>42.72</v>
+        <v>70.77</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v>7.65</v>
+        <v>11.59</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>18.83</v>
+        <v>13.81</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>0.19</v>
+        <v>0.55</v>
       </c>
       <c r="O17" s="33" t="n">
-        <v>0.26</v>
+        <v>0.7</v>
       </c>
       <c r="P17" s="47" t="n">
-        <v>-24.38</v>
-      </c>
-      <c r="Q17" s="33" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="R17" s="33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="S17" s="31" t="inlineStr">
+        <v>-21.07</v>
+      </c>
+      <c r="Q17" s="47" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="R17" s="47" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="S17" s="33" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="T17" s="33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="U17" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3288,7 +3384,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Europe ex UK UCITS ETF Distributing</t>
+          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -3297,54 +3393,60 @@
         </is>
       </c>
       <c r="C18" s="29" t="n">
-        <v>0.21</v>
+        <v>2.22</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>0.67</v>
+        <v>1.8</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="F18" s="46" t="n">
-        <v>-0.42</v>
+        <v>13.03</v>
+      </c>
+      <c r="F18" s="29" t="n">
+        <v>9.31</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>7.79</v>
+        <v>16.96</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>2.83</v>
+        <v>16.56</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>15.17</v>
+        <v>41.25</v>
       </c>
       <c r="J18" s="29" t="n">
-        <v>41.11</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="K18" s="29" t="n">
-        <v>55.53</v>
+        <v>42.65</v>
       </c>
       <c r="L18" s="29" t="n">
-        <v>9.65</v>
+        <v>7.64</v>
       </c>
       <c r="M18" s="29" t="n">
-        <v>14.94</v>
+        <v>18.83</v>
       </c>
       <c r="N18" s="29" t="n">
-        <v>0.38</v>
+        <v>0.19</v>
       </c>
       <c r="O18" s="29" t="n">
-        <v>0.51</v>
+        <v>0.26</v>
       </c>
       <c r="P18" s="46" t="n">
-        <v>-22.86</v>
-      </c>
-      <c r="Q18" s="29" t="n">
-        <v>4.23</v>
-      </c>
-      <c r="R18" s="29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="S18" s="27" t="inlineStr">
+        <v>-24.38</v>
+      </c>
+      <c r="Q18" s="46" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="R18" s="46" t="n">
+        <v>-2.59</v>
+      </c>
+      <c r="S18" s="29" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="T18" s="29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="U18" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3404,12 +3506,18 @@
         <v>-19.81</v>
       </c>
       <c r="Q19" s="47" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="R19" s="47" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="S19" s="47" t="n">
         <v>-6</v>
       </c>
-      <c r="R19" s="33" t="n">
+      <c r="T19" s="33" t="n">
         <v>0.02</v>
       </c>
-      <c r="S19" s="31" t="inlineStr">
+      <c r="U19" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3418,7 +3526,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>iShares VII PLC - iShares Nikkei 225 ETF JPY Acc</t>
+          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -3427,54 +3535,60 @@
         </is>
       </c>
       <c r="C20" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="D20" s="29" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="E20" s="29" t="n">
-        <v>9.6</v>
+        <v>0.31</v>
+      </c>
+      <c r="D20" s="46" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="E20" s="46" t="n">
+        <v>-1.11</v>
       </c>
       <c r="F20" s="29" t="n">
-        <v>10.93</v>
-      </c>
-      <c r="G20" s="29" t="n">
-        <v>10.3</v>
+        <v>0.9</v>
+      </c>
+      <c r="G20" s="46" t="n">
+        <v>-1.55</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="I20" s="29" t="n">
-        <v>44.84</v>
-      </c>
-      <c r="J20" s="29" t="n">
-        <v>73.92</v>
-      </c>
-      <c r="K20" s="29" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="L20" s="29" t="n">
-        <v>9.539999999999999</v>
+        <v>0.02</v>
+      </c>
+      <c r="I20" s="46" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="J20" s="46" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="K20" s="46" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="L20" s="46" t="n">
+        <v>-0.33</v>
       </c>
       <c r="M20" s="29" t="n">
-        <v>18.27</v>
-      </c>
-      <c r="N20" s="29" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="O20" s="29" t="n">
-        <v>0.46</v>
+        <v>10.65</v>
+      </c>
+      <c r="N20" s="46" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="O20" s="46" t="n">
+        <v>-0.61</v>
       </c>
       <c r="P20" s="46" t="n">
-        <v>-21.24</v>
-      </c>
-      <c r="Q20" s="29" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="R20" s="29" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="S20" s="27" t="inlineStr">
+        <v>-15.77</v>
+      </c>
+      <c r="Q20" s="46" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="R20" s="46" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="S20" s="46" t="n">
+        <v>-4.14</v>
+      </c>
+      <c r="T20" s="46" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="U20" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3483,7 +3597,7 @@
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t>iShares VII PLC - iShares Core S&amp;P 500 UCITS ETF</t>
+          <t>Vanguard FTSE Developed Europe ex UK UCITS ETF Distributing</t>
         </is>
       </c>
       <c r="B21" s="31" t="inlineStr">
@@ -3491,55 +3605,61 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C21" s="47" t="n">
-        <v>-0.1</v>
+      <c r="C21" s="33" t="n">
+        <v>0.21</v>
       </c>
       <c r="D21" s="33" t="n">
-        <v>1.15</v>
+        <v>0.67</v>
       </c>
       <c r="E21" s="33" t="n">
-        <v>8.83</v>
-      </c>
-      <c r="F21" s="33" t="n">
-        <v>5.42</v>
+        <v>4.89</v>
+      </c>
+      <c r="F21" s="47" t="n">
+        <v>-0.42</v>
       </c>
       <c r="G21" s="33" t="n">
-        <v>4.8</v>
+        <v>7.79</v>
       </c>
       <c r="H21" s="33" t="n">
-        <v>6.4</v>
+        <v>2.83</v>
       </c>
       <c r="I21" s="33" t="n">
-        <v>25.3</v>
+        <v>15.17</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>70.90000000000001</v>
+        <v>41.11</v>
       </c>
       <c r="K21" s="33" t="n">
-        <v>88.40000000000001</v>
+        <v>55.53</v>
       </c>
       <c r="L21" s="33" t="n">
-        <v>13.82</v>
+        <v>9.65</v>
       </c>
       <c r="M21" s="33" t="n">
-        <v>17.29</v>
+        <v>14.94</v>
       </c>
       <c r="N21" s="33" t="n">
-        <v>0.57</v>
+        <v>0.38</v>
       </c>
       <c r="O21" s="33" t="n">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
       <c r="P21" s="47" t="n">
-        <v>-22.73</v>
-      </c>
-      <c r="Q21" s="33" t="n">
-        <v>6.37</v>
-      </c>
-      <c r="R21" s="33" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="S21" s="31" t="inlineStr">
+        <v>-22.86</v>
+      </c>
+      <c r="Q21" s="47" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="R21" s="47" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="S21" s="33" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="T21" s="33" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="U21" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3548,7 +3668,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
+          <t>iShares VII PLC - iShares Core S&amp;P 500 UCITS ETF</t>
         </is>
       </c>
       <c r="B22" s="27" t="inlineStr">
@@ -3556,55 +3676,61 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C22" s="29" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="D22" s="46" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="E22" s="46" t="n">
-        <v>-1.11</v>
+      <c r="C22" s="46" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="D22" s="29" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>8.880000000000001</v>
       </c>
       <c r="F22" s="29" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G22" s="46" t="n">
-        <v>-1.55</v>
+        <v>5.47</v>
+      </c>
+      <c r="G22" s="29" t="n">
+        <v>4.85</v>
       </c>
       <c r="H22" s="29" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I22" s="46" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="J22" s="46" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="K22" s="46" t="n">
-        <v>-1.61</v>
-      </c>
-      <c r="L22" s="46" t="n">
-        <v>-0.33</v>
+        <v>6.45</v>
+      </c>
+      <c r="I22" s="29" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="J22" s="29" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="K22" s="29" t="n">
+        <v>88.48999999999999</v>
+      </c>
+      <c r="L22" s="29" t="n">
+        <v>13.84</v>
       </c>
       <c r="M22" s="29" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="N22" s="46" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="O22" s="46" t="n">
-        <v>-0.61</v>
+        <v>17.29</v>
+      </c>
+      <c r="N22" s="29" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="O22" s="29" t="n">
+        <v>0.79</v>
       </c>
       <c r="P22" s="46" t="n">
-        <v>-15.77</v>
+        <v>-22.73</v>
       </c>
       <c r="Q22" s="46" t="n">
-        <v>-4.14</v>
+        <v>-1.73</v>
       </c>
       <c r="R22" s="46" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="S22" s="27" t="inlineStr">
+        <v>-2.53</v>
+      </c>
+      <c r="S22" s="29" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="T22" s="29" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="U22" s="27" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3663,13 +3789,19 @@
       <c r="P23" s="47" t="n">
         <v>-15.94</v>
       </c>
-      <c r="Q23" s="33" t="n">
+      <c r="Q23" s="47" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="R23" s="47" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="S23" s="33" t="n">
         <v>17.05</v>
       </c>
-      <c r="R23" s="33" t="n">
+      <c r="T23" s="33" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="S23" s="31" t="inlineStr">
+      <c r="U23" s="31" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3690,263 +3822,313 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
           <t>● Strong</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>● Fair</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>● Weak</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="27" t="inlineStr">
         <is>
           <t>CAGR</t>
         </is>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B28" s="48" t="inlineStr">
+        <is>
+          <t>Compound Annual Growth Rate. The single yearly return that, if repeated every year, would grow your portfolio from start to end value. Accounts for compounding. ~7% is the long-term global equity average.</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
         <is>
           <t>&gt; 7.0</t>
         </is>
       </c>
-      <c r="C28" s="27" t="inlineStr">
+      <c r="D28" s="27" t="inlineStr">
         <is>
           <t>3.0 – 7.0</t>
         </is>
       </c>
-      <c r="D28" s="27" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>&lt; 3.0</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="F28" s="27" t="inlineStr">
         <is>
           <t>Equity risk premium (Dimson et al.)</t>
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="48" customHeight="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>α (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Extra annual return vs the benchmark, after adjusting for how risky the portfolio is (CAPM). Positive = you beat the market beyond what your risk alone justified. Negative = you underperformed after fees and noise.</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
         <is>
           <t>&gt; 0.0</t>
         </is>
       </c>
-      <c r="C29" s="31" t="inlineStr">
+      <c r="D29" s="31" t="inlineStr">
         <is>
           <t>-1.0 – 0.0</t>
         </is>
       </c>
-      <c r="D29" s="31" t="inlineStr">
+      <c r="E29" s="31" t="inlineStr">
         <is>
           <t>&lt; -1.0</t>
         </is>
       </c>
-      <c r="E29" s="31" t="inlineStr">
+      <c r="F29" s="31" t="inlineStr">
         <is>
           <t>Jensen's Alpha (CAPM)</t>
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="27" t="inlineStr">
         <is>
           <t>β (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="B30" s="27" t="inlineStr">
+      <c r="B30" s="48" t="inlineStr">
+        <is>
+          <t>How much your portfolio moves when the benchmark moves 1%. β=1 in line, β=0.5 half as reactive, β=1.5 amplifies by 50%, β≈0 uncorrelated. Tells you how much systematic market risk you're running.</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
         <is>
           <t>&lt; 0.7%</t>
         </is>
       </c>
-      <c r="C30" s="27" t="inlineStr">
+      <c r="D30" s="27" t="inlineStr">
         <is>
           <t>1.0% – 0.7%</t>
         </is>
       </c>
-      <c r="D30" s="27" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>&gt; 1.0%</t>
         </is>
       </c>
-      <c r="E30" s="27" t="inlineStr">
+      <c r="F30" s="27" t="inlineStr">
         <is>
           <t>CAPM, 1.0 = market</t>
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Max DD</t>
         </is>
       </c>
-      <c r="B31" s="31" t="inlineStr">
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Maximum Drawdown. Worst peak-to-trough loss over the period — the most painful scenario an investor lived through. -20% is typical for diversified equity; deeper drops signal concentration or high volatility.</t>
+        </is>
+      </c>
+      <c r="C31" s="31" t="inlineStr">
         <is>
           <t>&lt; 15.0%</t>
         </is>
       </c>
-      <c r="C31" s="31" t="inlineStr">
+      <c r="D31" s="31" t="inlineStr">
         <is>
           <t>30.0% – 15.0%</t>
         </is>
       </c>
-      <c r="D31" s="31" t="inlineStr">
+      <c r="E31" s="31" t="inlineStr">
         <is>
           <t>&gt; 30.0%</t>
         </is>
       </c>
-      <c r="E31" s="31" t="inlineStr">
+      <c r="F31" s="31" t="inlineStr">
         <is>
           <t>Retail drawdown tolerance</t>
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="48" customHeight="1">
       <c r="A32" s="27" t="inlineStr">
         <is>
           <t>Volatility</t>
         </is>
       </c>
-      <c r="B32" s="27" t="inlineStr">
+      <c r="B32" s="48" t="inlineStr">
+        <is>
+          <t>How bumpy the ride is. Annualized standard deviation of daily returns. A 15% vol means ~±15% year-to-year noise around the average return. Equity indexes ~15–20%, bonds ~3–7%.</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
         <is>
           <t>&lt; 10.0%</t>
         </is>
       </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="D32" s="27" t="inlineStr">
         <is>
           <t>18.0% – 10.0%</t>
         </is>
       </c>
-      <c r="D32" s="27" t="inlineStr">
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>&gt; 18.0%</t>
         </is>
       </c>
-      <c r="E32" s="27" t="inlineStr">
+      <c r="F32" s="27" t="inlineStr">
         <is>
           <t>Hist. equity vol ~15%</t>
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>Sharpe</t>
         </is>
       </c>
-      <c r="B33" s="31" t="inlineStr">
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Return per unit of risk taken: (CAGR − risk-free rate) / Volatility. Above 1 is good, above 2 is excellent, negative means you were paid less than a safe bond for the risk you ran.</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="inlineStr">
         <is>
           <t>&gt; 1.0</t>
         </is>
       </c>
-      <c r="C33" s="31" t="inlineStr">
+      <c r="D33" s="31" t="inlineStr">
         <is>
           <t>0.5 – 1.0</t>
         </is>
       </c>
-      <c r="D33" s="31" t="inlineStr">
+      <c r="E33" s="31" t="inlineStr">
         <is>
           <t>&lt; 0.5</t>
         </is>
       </c>
-      <c r="E33" s="31" t="inlineStr">
+      <c r="F33" s="31" t="inlineStr">
         <is>
           <t>Sharpe (1994)</t>
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="48" customHeight="1">
       <c r="A34" s="27" t="inlineStr">
         <is>
           <t>Sortino</t>
         </is>
       </c>
-      <c r="B34" s="27" t="inlineStr">
+      <c r="B34" s="48" t="inlineStr">
+        <is>
+          <t>Like Sharpe but only penalizes downside volatility (ignores upside swings). More honest when returns are asymmetric. Usually higher than Sharpe — the gap shows how much of your volatility is actually good volatility.</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
         <is>
           <t>&gt; 1.5</t>
         </is>
       </c>
-      <c r="C34" s="27" t="inlineStr">
+      <c r="D34" s="27" t="inlineStr">
         <is>
           <t>0.7 – 1.5</t>
         </is>
       </c>
-      <c r="D34" s="27" t="inlineStr">
+      <c r="E34" s="27" t="inlineStr">
         <is>
           <t>&lt; 0.7</t>
         </is>
       </c>
-      <c r="E34" s="27" t="inlineStr">
+      <c r="F34" s="27" t="inlineStr">
         <is>
           <t>Sortino &amp; Price (1994)</t>
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="48" customHeight="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>VaR 95%</t>
         </is>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Value at Risk. The daily loss exceeded only 5% of the time (historical simulation). A VaR of -1.2% means on an average month you should expect about one day worse than -1.2%. Non-parametric: no normal-distribution assumption.</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
         <is>
           <t>&lt; 0.8%</t>
         </is>
       </c>
-      <c r="C35" s="31" t="inlineStr">
+      <c r="D35" s="31" t="inlineStr">
         <is>
           <t>1.5% – 0.8%</t>
         </is>
       </c>
-      <c r="D35" s="31" t="inlineStr">
+      <c r="E35" s="31" t="inlineStr">
         <is>
           <t>&gt; 1.5%</t>
         </is>
       </c>
-      <c r="E35" s="31" t="inlineStr">
+      <c r="F35" s="31" t="inlineStr">
         <is>
           <t>Basel III (retail adj.)</t>
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="48" customHeight="1">
       <c r="A36" s="27" t="inlineStr">
         <is>
           <t>CVaR 95%</t>
         </is>
       </c>
-      <c r="B36" s="27" t="inlineStr">
+      <c r="B36" s="48" t="inlineStr">
+        <is>
+          <t>Conditional VaR, a.k.a. Expected Shortfall. The average loss on the worst 5% of days. Always more negative than VaR. Captures tail risk VaR misses — how bad it really gets when it goes bad.</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>&lt; 1.2%</t>
         </is>
       </c>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="D36" s="27" t="inlineStr">
         <is>
           <t>2.0% – 1.2%</t>
         </is>
       </c>
-      <c r="D36" s="27" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>&gt; 2.0%</t>
         </is>
       </c>
-      <c r="E36" s="27" t="inlineStr">
+      <c r="F36" s="27" t="inlineStr">
         <is>
           <t>Artzner et al. (1999)</t>
         </is>
@@ -3955,13 +4137,13 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 09:47 v2.0</t>
+          <t>Generated 2026-05-04 10:02 v2.0</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A2:U2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4050,13 +4232,13 @@
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>14.26779706186569</v>
+        <v>14.26530952530278</v>
       </c>
       <c r="E5" s="29" t="n">
         <v>415.5184553004801</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>59.28532995687162</v>
+        <v>59.27499378337036</v>
       </c>
     </row>
     <row r="6">
@@ -4076,13 +4258,13 @@
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>13.23905143133624</v>
+        <v>13.23674325269094</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>91.33928843906948</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>12.09245537346497</v>
+        <v>12.09034709951444</v>
       </c>
     </row>
     <row r="7">
@@ -4102,13 +4284,13 @@
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>8.460803908866717</v>
+        <v>8.459328799641117</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>55.27743647935755</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>4.6769155063668</v>
+        <v>4.676100103801618</v>
       </c>
     </row>
     <row r="8">
@@ -4128,13 +4310,13 @@
         </is>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.3624886227922</v>
+        <v>15.36969361005393</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>21.42187356948853</v>
+        <v>21.50000333786011</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>3.290932889901604</v>
+        <v>3.304484639180467</v>
       </c>
     </row>
     <row r="9">
@@ -4154,13 +4336,13 @@
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>8.505512682692782</v>
+        <v>8.500249996866843</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>36.58571243286133</v>
+        <v>36.52500425066267</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>3.11180241103053</v>
+        <v>3.104716672672568</v>
       </c>
     </row>
     <row r="10">
@@ -4180,13 +4362,13 @@
         </is>
       </c>
       <c r="D10" s="33" t="n">
-        <v>7.041964251641569</v>
+        <v>7.040736511754693</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>43.92423918752959</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>3.093129221391371</v>
+        <v>3.092589945986859</v>
       </c>
     </row>
     <row r="11">
@@ -4206,13 +4388,13 @@
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>7.344315367508301</v>
+        <v>7.343034913845621</v>
       </c>
       <c r="E11" s="29" t="n">
         <v>41.5263607345748</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>3.04982689299631</v>
+        <v>3.049295167189306</v>
       </c>
     </row>
     <row r="12">
@@ -4232,13 +4414,13 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>12.31012766337849</v>
+        <v>12.31375315772519</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>16.52839220992303</v>
+        <v>16.58303716504107</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.03466618174543</v>
+        <v>2.041994262556988</v>
       </c>
     </row>
     <row r="13">
@@ -4258,13 +4440,13 @@
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>7.290126950746573</v>
+        <v>7.294415251161368</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>20.41326250348772</v>
+        <v>20.50510328643176</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>1.488152751293403</v>
+        <v>1.495727381391869</v>
       </c>
     </row>
     <row r="14">
@@ -4284,7 +4466,7 @@
         </is>
       </c>
       <c r="D14" s="33" t="n">
-        <v>6.177812059171433</v>
+        <v>6.176734980957511</v>
       </c>
       <c r="E14" s="33" t="n">
         <v>0</v>
@@ -4329,10 +4511,10 @@
         </is>
       </c>
       <c r="B18" s="28" t="n">
-        <v>52427.96042730808</v>
+        <v>52442.07356523337</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>92.39865586729506</v>
+        <v>92.42597375466755</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>6</v>
@@ -4417,10 +4599,10 @@
         </is>
       </c>
       <c r="B25" s="29" t="n">
-        <v>41.75790478337835</v>
+        <v>41.77116920492907</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>19.45450942763309</v>
+        <v>19.52938126311098</v>
       </c>
     </row>
     <row r="26">
@@ -4430,10 +4612,10 @@
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>15.53026313713126</v>
+        <v>15.5217931241751</v>
       </c>
       <c r="C26" s="33" t="n">
-        <v>29.00379300117493</v>
+        <v>29.01250379426139</v>
       </c>
     </row>
     <row r="27">
@@ -4443,10 +4625,10 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>10.66366665568281</v>
+        <v>10.66269639765878</v>
       </c>
       <c r="C27" s="29" t="n">
-        <v>28.58645842016861</v>
+        <v>28.64311527060715</v>
       </c>
     </row>
     <row r="28">
@@ -4456,10 +4638,10 @@
         </is>
       </c>
       <c r="B28" s="33" t="n">
-        <v>24.1498199211525</v>
+        <v>24.14476795526446</v>
       </c>
       <c r="C28" s="33" t="n">
-        <v>152.4511971244854</v>
+        <v>152.507853974924</v>
       </c>
     </row>
     <row r="29">
@@ -4469,10 +4651,10 @@
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>7.898345502655069</v>
+        <v>7.899573317972592</v>
       </c>
       <c r="C29" s="29" t="n">
-        <v>28.58645842016861</v>
+        <v>28.64311527060715</v>
       </c>
     </row>
   </sheetData>
@@ -4525,12 +4707,12 @@
           <t>Total Value (EUR)</t>
         </is>
       </c>
-      <c r="B4" s="48" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>Sum of current market values of all holdings, converted to EUR.</t>
         </is>
       </c>
-      <c r="C4" s="48" t="inlineStr">
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Point-in-time (today)</t>
         </is>
@@ -4542,12 +4724,12 @@
           <t>YTD Return</t>
         </is>
       </c>
-      <c r="B5" s="49" t="inlineStr">
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Year-to-date return. Formula: (Current Value / Value at Jan 1) - 1.</t>
         </is>
       </c>
-      <c r="C5" s="49" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Jan 1 of current year to today</t>
         </is>
@@ -4559,12 +4741,12 @@
           <t>CAGR</t>
         </is>
       </c>
-      <c r="B6" s="48" t="inlineStr">
+      <c r="B6" s="50" t="inlineStr">
         <is>
           <t>Compound Annual Growth Rate. Formula: (End/Start)^(1/years) - 1. Measures mean annual growth rate assuming constant compounding.</t>
         </is>
       </c>
-      <c r="C6" s="48" t="inlineStr">
+      <c r="C6" s="50" t="inlineStr">
         <is>
           <t>Full history: 2.3 years (853 calendar days)</t>
         </is>
@@ -4576,12 +4758,12 @@
           <t>Sharpe Ratio</t>
         </is>
       </c>
-      <c r="B7" s="49" t="inlineStr">
+      <c r="B7" s="51" t="inlineStr">
         <is>
           <t>Risk-adjusted return. Formula: (Return - Rf) / Volatility. Higher is better.</t>
         </is>
       </c>
-      <c r="C7" s="49" t="inlineStr">
+      <c r="C7" s="51" t="inlineStr">
         <is>
           <t>Risk-free rate: 4.0%. Period: 2.3 years (853 calendar days)</t>
         </is>
@@ -4593,12 +4775,12 @@
           <t>Sortino Ratio</t>
         </is>
       </c>
-      <c r="B8" s="48" t="inlineStr">
+      <c r="B8" s="50" t="inlineStr">
         <is>
           <t>Downside risk-adjusted return. Uses only negative returns for deviation. Formula: (Return - Rf) / Downside Deviation.</t>
         </is>
       </c>
-      <c r="C8" s="48" t="inlineStr">
+      <c r="C8" s="50" t="inlineStr">
         <is>
           <t>Risk-free rate: 4.0%. Period: 2.3 years (853 calendar days)</t>
         </is>
@@ -4610,12 +4792,12 @@
           <t>Volatility</t>
         </is>
       </c>
-      <c r="B9" s="49" t="inlineStr">
+      <c r="B9" s="51" t="inlineStr">
         <is>
           <t>Annualized std dev of daily returns. Formula: StdDev(daily) x sqrt(252).</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="51" t="inlineStr">
         <is>
           <t>Period: 2.3 years (853 calendar days). Trading days/year: 252</t>
         </is>
@@ -4627,12 +4809,12 @@
           <t>Max Drawdown</t>
         </is>
       </c>
-      <c r="B10" s="48" t="inlineStr">
+      <c r="B10" s="50" t="inlineStr">
         <is>
           <t>Largest peak-to-trough decline. Formula: min((V - CumMax) / CumMax).</t>
         </is>
       </c>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="C10" s="50" t="inlineStr">
         <is>
           <t>Period: 2.3 years (853 calendar days)</t>
         </is>
@@ -4644,12 +4826,12 @@
           <t>VaR (95%)</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="51" t="inlineStr">
         <is>
           <t>Value at Risk via historical simulation. The 5th percentile of daily returns. Non-parametric: no distributional assumptions, robust for fat tails.</t>
         </is>
       </c>
-      <c r="C11" s="49" t="inlineStr">
+      <c r="C11" s="51" t="inlineStr">
         <is>
           <t>Period: 2.3 years (853 calendar days). Confidence: 95%</t>
         </is>
@@ -4661,12 +4843,12 @@
           <t>CVaR (95%)</t>
         </is>
       </c>
-      <c r="B12" s="48" t="inlineStr">
+      <c r="B12" s="50" t="inlineStr">
         <is>
           <t>Conditional VaR (Expected Shortfall). Average loss beyond VaR threshold. A coherent risk measure per Artzner et al. (1999), preferred for tail risk.</t>
         </is>
       </c>
-      <c r="C12" s="48" t="inlineStr">
+      <c r="C12" s="50" t="inlineStr">
         <is>
           <t>Period: 2.3 years (853 calendar days). Confidence: 95%</t>
         </is>
@@ -4678,12 +4860,12 @@
           <t>Beta</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="51" t="inlineStr">
         <is>
           <t>CAPM sensitivity to market. Formula: Cov(Rp, Rb) / Var(Rb). Beta=1 means same as market.</t>
         </is>
       </c>
-      <c r="C13" s="49" t="inlineStr">
+      <c r="C13" s="51" t="inlineStr">
         <is>
           <t>Benchmark: S&amp;P 500. Period: 2.3 years (853 calendar days)</t>
         </is>
@@ -4695,12 +4877,12 @@
           <t>Alpha</t>
         </is>
       </c>
-      <c r="B14" s="48" t="inlineStr">
+      <c r="B14" s="50" t="inlineStr">
         <is>
           <t>Jensen's Alpha. Excess return vs CAPM expected. Formula: Rp - [Rf + Beta x (Rb - Rf)].</t>
         </is>
       </c>
-      <c r="C14" s="48" t="inlineStr">
+      <c r="C14" s="50" t="inlineStr">
         <is>
           <t>Benchmark: S&amp;P 500. Risk-free rate: 4.0%</t>
         </is>
@@ -4712,12 +4894,12 @@
           <t>Weighted Yield</t>
         </is>
       </c>
-      <c r="B15" s="49" t="inlineStr">
+      <c r="B15" s="51" t="inlineStr">
         <is>
           <t>Portfolio-weighted average dividend/coupon yield.</t>
         </is>
       </c>
-      <c r="C15" s="49" t="inlineStr">
+      <c r="C15" s="51" t="inlineStr">
         <is>
           <t>Based on latest yield data from yfinance</t>
         </is>
@@ -4729,12 +4911,12 @@
           <t>Geography Allocation</t>
         </is>
       </c>
-      <c r="B16" s="48" t="inlineStr">
+      <c r="B16" s="50" t="inlineStr">
         <is>
           <t>Geographic exposure of equity holdings only. Multi-geo ETFs split proportionally.</t>
         </is>
       </c>
-      <c r="C16" s="48" t="inlineStr">
+      <c r="C16" s="50" t="inlineStr">
         <is>
           <t>Equity only. Sources: justETF, index_geo_allocation.csv, yfinance</t>
         </is>
@@ -4746,12 +4928,12 @@
           <t>Rebalancing Amount</t>
         </is>
       </c>
-      <c r="B17" s="49" t="inlineStr">
+      <c r="B17" s="51" t="inlineStr">
         <is>
           <t>Suggested trade amount to reach target. Asset class: total value. Geography: equity value.</t>
         </is>
       </c>
-      <c r="C17" s="49" t="inlineStr">
+      <c r="C17" s="51" t="inlineStr">
         <is>
           <t>Threshold from config (rebalancing_threshold)</t>
         </is>
@@ -4760,7 +4942,7 @@
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 09:47 v2.0</t>
+          <t>Generated 2026-05-04 10:02 v2.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel): respect per-metric unit in Legend thresholds
Beta, Sharpe, and Sortino are pure ratios, not percentages. The legend
previously printed '< 0.7%' for Beta because the invert-branch always
appended '%'. Add an optional 'unit' key to metric_ratings in
constants.yaml (default empty) and format thresholds with that unit.

- Ratio metrics (beta, sharpe, sortino) → no unit suffix
- Percentage metrics (cagr, alpha, max_drawdown, volatility, var_pct,
  cvar_pct) → '%' suffix, now applied consistently to both strong/fair/
  weak columns regardless of invert direction.

Regenerate the sample dashboard with the corrected legend.
</commit_message>
<xml_diff>
--- a/output/sample/portfolio_dashboard_sample.xlsx
+++ b/output/sample/portfolio_dashboard_sample.xlsx
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>80948.91581741307</v>
+        <v>80950.0840273767</v>
       </c>
       <c r="D5" s="2" t="n"/>
     </row>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>26808.91581741307</v>
+        <v>26810.0840273767</v>
       </c>
       <c r="D6" s="2" t="n"/>
     </row>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>49.5177610221889</v>
+        <v>49.51991877978703</v>
       </c>
       <c r="D7" s="2" t="n"/>
     </row>
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>64.78415805286481</v>
+        <v>64.7846662610765</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>65</v>
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>41.77116920492907</v>
+        <v>41.77246629294275</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>55</v>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>20.57977816653656</v>
+        <v>20.57948117485098</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>25</v>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>24.14476795526446</v>
+        <v>24.14423011363721</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>8</v>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>8.459328799641117</v>
+        <v>8.459206721050242</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>5</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="F14" s="22" t="n">
-        <v>15.5217931241751</v>
+        <v>15.52144736535534</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>11</v>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>6.176734980957511</v>
+        <v>6.176645843022274</v>
       </c>
       <c r="C15" s="18" t="n">
         <v>5</v>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="F15" s="17" t="n">
-        <v>10.66269639765878</v>
+        <v>10.66245887862393</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>14</v>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F16" s="22" t="n">
-        <v>7.899573317972592</v>
+        <v>7.899397349440786</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>12</v>
@@ -1063,7 +1063,7 @@
         <v>12441.60034179688</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>15.36969361005393</v>
+        <v>15.36947180634083</v>
       </c>
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="12" t="inlineStr">
@@ -1082,7 +1082,7 @@
         <v>11547.61339873075</v>
       </c>
       <c r="C22" s="33" t="n">
-        <v>14.26530952530278</v>
+        <v>14.26510365921972</v>
       </c>
       <c r="D22" s="30" t="n"/>
       <c r="E22" s="34" t="inlineStr">
@@ -1101,7 +1101,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="C23" s="29" t="n">
-        <v>13.23674325269094</v>
+        <v>13.236552230093</v>
       </c>
       <c r="D23" s="30" t="n"/>
       <c r="E23" s="35" t="inlineStr">
@@ -1117,10 +1117,10 @@
         </is>
       </c>
       <c r="B24" s="32" t="n">
-        <v>9967.849677611011</v>
+        <v>9969.017887574628</v>
       </c>
       <c r="C24" s="33" t="n">
-        <v>12.31375315772519</v>
+        <v>12.3150185788605</v>
       </c>
       <c r="D24" s="30" t="n"/>
       <c r="E24" s="34" t="inlineStr">
@@ -1139,7 +1139,7 @@
         <v>6880.860214233398</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>8.500249996866843</v>
+        <v>8.500127327732415</v>
       </c>
       <c r="D25" s="30" t="n"/>
       <c r="E25" s="12" t="inlineStr">
@@ -1154,7 +1154,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 10:02 v2.0</t>
+          <t>Generated 2026-05-04 10:06 v2.0</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 10:02 v2.0</t>
+          <t>Generated 2026-05-04 10:06 v2.0</t>
         </is>
       </c>
     </row>
@@ -1549,10 +1549,10 @@
         <v>12441.60034179688</v>
       </c>
       <c r="L4" s="29" t="n">
-        <v>15.36969361005393</v>
+        <v>15.36947180634083</v>
       </c>
       <c r="M4" s="29" t="n">
-        <v>23.72446300453892</v>
+        <v>23.723934525499</v>
       </c>
       <c r="N4" s="28" t="n">
         <v>2201.600341796875</v>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="S4" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -1628,10 +1628,10 @@
         <v>11547.61339873075</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>14.26530952530278</v>
+        <v>14.26510365921972</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>22.01974981856225</v>
+        <v>22.01925931320324</v>
       </c>
       <c r="N5" s="32" t="n">
         <v>9307.613398730755</v>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="S5" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -1698,25 +1698,25 @@
         <v>570</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>664.5233118407341</v>
+        <v>664.6011925049752</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>8550</v>
       </c>
       <c r="K6" s="28" t="n">
-        <v>9967.849677611011</v>
+        <v>9969.017887574628</v>
       </c>
       <c r="L6" s="29" t="n">
-        <v>12.31375315772519</v>
+        <v>12.3150185788605</v>
       </c>
       <c r="M6" s="29" t="n">
-        <v>19.00735230313095</v>
+        <v>19.00915647111936</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>1417.849677611011</v>
+        <v>1419.017887574628</v>
       </c>
       <c r="O6" s="29" t="n">
-        <v>16.58303716504107</v>
+        <v>16.59670043946933</v>
       </c>
       <c r="P6" s="27" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -1786,10 +1786,10 @@
         <v>6880.860214233398</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>8.500249996866843</v>
+        <v>8.500127327732415</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>13.12087746811576</v>
+        <v>13.12058519137484</v>
       </c>
       <c r="N7" s="32" t="n">
         <v>1840.860214233398</v>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="S7" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -1865,10 +1865,10 @@
         <v>5904.750061035156</v>
       </c>
       <c r="L8" s="29" t="n">
-        <v>7.294415251161368</v>
+        <v>7.294309983715664</v>
       </c>
       <c r="M8" s="29" t="n">
-        <v>11.25956633596908</v>
+        <v>11.25931552123806</v>
       </c>
       <c r="N8" s="28" t="n">
         <v>1004.750061035156</v>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="S8" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -1944,10 +1944,10 @@
         <v>5699.399871826172</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v>7.040736511754693</v>
+        <v>7.04063490520736</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v>10.86799106968304</v>
+        <v>10.8677489775655</v>
       </c>
       <c r="N9" s="32" t="n">
         <v>1739.399871826172</v>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="S9" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="L10" s="29" t="n">
-        <v>13.23674325269094</v>
+        <v>13.236552230093</v>
       </c>
       <c r="M10" s="29" t="n">
         <v>64.31917363528412</v>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="S10" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
         <v>5944.107150852142</v>
       </c>
       <c r="L11" s="33" t="n">
-        <v>7.343034913845621</v>
+        <v>7.34292894475797</v>
       </c>
       <c r="M11" s="33" t="n">
         <v>35.68082636471589</v>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="S11" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 10:01</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
         <v>5000</v>
       </c>
       <c r="L12" s="29" t="n">
-        <v>6.176734980957511</v>
+        <v>6.176645843022274</v>
       </c>
       <c r="M12" s="29" t="n">
         <v>100</v>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="S12" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 10:02</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
         <v>6847.734948739668</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v>8.459328799641117</v>
+        <v>8.459206721050242</v>
       </c>
       <c r="M13" s="33" t="n">
         <v>100</v>
@@ -2288,14 +2288,14 @@
       </c>
       <c r="S13" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 10:02</t>
+          <t>2026-05-04 10:06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 10:02 v2.0</t>
+          <t>Generated 2026-05-04 10:06 v2.0</t>
         </is>
       </c>
     </row>
@@ -2612,31 +2612,31 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>6.61</v>
+        <v>6.63</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>4.44</v>
+        <v>4.45</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>6.36</v>
+        <v>6.37</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>6.49</v>
+        <v>6.51</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>23.65</v>
+        <v>23.67</v>
       </c>
       <c r="J7" s="33" t="n">
-        <v>56.12</v>
+        <v>56.14</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>58.7</v>
+        <v>58.72</v>
       </c>
       <c r="L7" s="33" t="n">
         <v>9.83</v>
@@ -2660,7 +2660,7 @@
         <v>-2.13</v>
       </c>
       <c r="S7" s="47" t="n">
-        <v>-0.5</v>
+        <v>-0.49</v>
       </c>
       <c r="T7" s="33" t="n">
         <v>0.78</v>
@@ -2824,35 +2824,35 @@
           <t>Benchmark index</t>
         </is>
       </c>
-      <c r="C10" s="46" t="n">
-        <v>-0.01</v>
+      <c r="C10" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>5.94</v>
+        <v>5.95</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>3.95</v>
+        <v>3.96</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>5.05</v>
+        <v>5.07</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>5.34</v>
+        <v>5.35</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>21.71</v>
+        <v>21.72</v>
       </c>
       <c r="J10" s="29" t="n">
-        <v>55.65</v>
+        <v>55.67</v>
       </c>
       <c r="K10" s="29" t="n">
-        <v>63.25</v>
+        <v>63.27</v>
       </c>
       <c r="L10" s="29" t="n">
-        <v>10.46</v>
+        <v>10.47</v>
       </c>
       <c r="M10" s="29" t="n">
         <v>16.47</v>
@@ -3242,7 +3242,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>iShares VII PLC - iShares Nikkei 225 ETF JPY Acc</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
@@ -3251,58 +3251,58 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.04</v>
+        <v>1.01</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.93</v>
+        <v>1.32</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>9.6</v>
+        <v>8.06</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>10.93</v>
+        <v>5.01</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>10.3</v>
+        <v>6.92</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>17.9</v>
+        <v>7.15</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>44.84</v>
+        <v>24.98</v>
       </c>
       <c r="J16" s="29" t="n">
-        <v>73.92</v>
+        <v>63.28</v>
       </c>
       <c r="K16" s="29" t="n">
-        <v>57.6</v>
+        <v>70.77</v>
       </c>
       <c r="L16" s="29" t="n">
-        <v>9.539999999999999</v>
+        <v>11.59</v>
       </c>
       <c r="M16" s="29" t="n">
-        <v>18.27</v>
+        <v>13.81</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.3</v>
+        <v>0.55</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.46</v>
+        <v>0.7</v>
       </c>
       <c r="P16" s="46" t="n">
-        <v>-21.24</v>
+        <v>-21.07</v>
       </c>
       <c r="Q16" s="46" t="n">
-        <v>-1.78</v>
+        <v>-1.39</v>
       </c>
       <c r="R16" s="46" t="n">
-        <v>-2.5</v>
+        <v>-2.13</v>
       </c>
       <c r="S16" s="29" t="n">
-        <v>3.42</v>
+        <v>5.98</v>
       </c>
       <c r="T16" s="29" t="n">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="U16" s="27" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B17" s="31" t="inlineStr">
@@ -3322,58 +3322,58 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>1.01</v>
+        <v>2.22</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>1.32</v>
+        <v>1.8</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>8.06</v>
+        <v>13.03</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>5.01</v>
+        <v>9.31</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>6.92</v>
+        <v>16.96</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>7.15</v>
+        <v>16.56</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>24.98</v>
+        <v>41.25</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>63.28</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>70.77</v>
+        <v>42.65</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v>11.59</v>
+        <v>7.64</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>13.81</v>
+        <v>18.83</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>0.55</v>
+        <v>0.19</v>
       </c>
       <c r="O17" s="33" t="n">
-        <v>0.7</v>
+        <v>0.26</v>
       </c>
       <c r="P17" s="47" t="n">
-        <v>-21.07</v>
+        <v>-24.38</v>
       </c>
       <c r="Q17" s="47" t="n">
-        <v>-1.39</v>
+        <v>-1.59</v>
       </c>
       <c r="R17" s="47" t="n">
-        <v>-2.13</v>
+        <v>-2.59</v>
       </c>
       <c r="S17" s="33" t="n">
-        <v>5.98</v>
+        <v>2.82</v>
       </c>
       <c r="T17" s="33" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="U17" s="31" t="inlineStr">
         <is>
@@ -3384,7 +3384,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
+          <t>Vanguard FTSE Developed Europe ex UK UCITS ETF Distributing</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -3393,58 +3393,58 @@
         </is>
       </c>
       <c r="C18" s="29" t="n">
-        <v>2.22</v>
+        <v>0.21</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>1.8</v>
+        <v>0.67</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>13.03</v>
-      </c>
-      <c r="F18" s="29" t="n">
-        <v>9.31</v>
+        <v>4.89</v>
+      </c>
+      <c r="F18" s="46" t="n">
+        <v>-0.42</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>16.96</v>
+        <v>7.79</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>16.56</v>
+        <v>2.83</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>41.25</v>
+        <v>15.17</v>
       </c>
       <c r="J18" s="29" t="n">
-        <v>69.29000000000001</v>
+        <v>41.11</v>
       </c>
       <c r="K18" s="29" t="n">
-        <v>42.65</v>
+        <v>55.53</v>
       </c>
       <c r="L18" s="29" t="n">
-        <v>7.64</v>
+        <v>9.65</v>
       </c>
       <c r="M18" s="29" t="n">
-        <v>18.83</v>
+        <v>14.94</v>
       </c>
       <c r="N18" s="29" t="n">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="O18" s="29" t="n">
-        <v>0.26</v>
+        <v>0.51</v>
       </c>
       <c r="P18" s="46" t="n">
-        <v>-24.38</v>
+        <v>-22.86</v>
       </c>
       <c r="Q18" s="46" t="n">
-        <v>-1.59</v>
+        <v>-1.53</v>
       </c>
       <c r="R18" s="46" t="n">
-        <v>-2.59</v>
+        <v>-2.22</v>
       </c>
       <c r="S18" s="29" t="n">
-        <v>2.82</v>
+        <v>4.23</v>
       </c>
       <c r="T18" s="29" t="n">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="U18" s="27" t="inlineStr">
         <is>
@@ -3526,7 +3526,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
+          <t>iShares VII PLC - iShares Nikkei 225 ETF JPY Acc</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -3535,58 +3535,58 @@
         </is>
       </c>
       <c r="C20" s="29" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="D20" s="46" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="E20" s="46" t="n">
-        <v>-1.11</v>
+        <v>0.04</v>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>9.6</v>
       </c>
       <c r="F20" s="29" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G20" s="46" t="n">
-        <v>-1.55</v>
+        <v>10.93</v>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>10.3</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I20" s="46" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="J20" s="46" t="n">
-        <v>-0.82</v>
-      </c>
-      <c r="K20" s="46" t="n">
-        <v>-1.61</v>
-      </c>
-      <c r="L20" s="46" t="n">
-        <v>-0.33</v>
+        <v>17.9</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>44.84</v>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>73.92</v>
+      </c>
+      <c r="K20" s="29" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="L20" s="29" t="n">
+        <v>9.539999999999999</v>
       </c>
       <c r="M20" s="29" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="N20" s="46" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="O20" s="46" t="n">
-        <v>-0.61</v>
+        <v>18.27</v>
+      </c>
+      <c r="N20" s="29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O20" s="29" t="n">
+        <v>0.46</v>
       </c>
       <c r="P20" s="46" t="n">
-        <v>-15.77</v>
+        <v>-21.24</v>
       </c>
       <c r="Q20" s="46" t="n">
-        <v>-1.1</v>
+        <v>-1.78</v>
       </c>
       <c r="R20" s="46" t="n">
-        <v>-1.48</v>
-      </c>
-      <c r="S20" s="46" t="n">
-        <v>-4.14</v>
-      </c>
-      <c r="T20" s="46" t="n">
-        <v>-0.02</v>
+        <v>-2.5</v>
+      </c>
+      <c r="S20" s="29" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="T20" s="29" t="n">
+        <v>0.26</v>
       </c>
       <c r="U20" s="27" t="inlineStr">
         <is>
@@ -3597,7 +3597,7 @@
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t>Vanguard FTSE Developed Europe ex UK UCITS ETF Distributing</t>
+          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B21" s="31" t="inlineStr">
@@ -3606,58 +3606,58 @@
         </is>
       </c>
       <c r="C21" s="33" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="D21" s="33" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="F21" s="47" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="G21" s="33" t="n">
-        <v>7.79</v>
+        <v>0.31</v>
+      </c>
+      <c r="D21" s="47" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="E21" s="47" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="F21" s="33" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G21" s="47" t="n">
+        <v>-1.55</v>
       </c>
       <c r="H21" s="33" t="n">
-        <v>2.83</v>
-      </c>
-      <c r="I21" s="33" t="n">
-        <v>15.17</v>
-      </c>
-      <c r="J21" s="33" t="n">
-        <v>41.11</v>
-      </c>
-      <c r="K21" s="33" t="n">
-        <v>55.53</v>
-      </c>
-      <c r="L21" s="33" t="n">
-        <v>9.65</v>
+        <v>0.02</v>
+      </c>
+      <c r="I21" s="47" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="J21" s="47" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="K21" s="47" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="L21" s="47" t="n">
+        <v>-0.33</v>
       </c>
       <c r="M21" s="33" t="n">
-        <v>14.94</v>
-      </c>
-      <c r="N21" s="33" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="O21" s="33" t="n">
-        <v>0.51</v>
+        <v>10.65</v>
+      </c>
+      <c r="N21" s="47" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="O21" s="47" t="n">
+        <v>-0.61</v>
       </c>
       <c r="P21" s="47" t="n">
-        <v>-22.86</v>
+        <v>-15.77</v>
       </c>
       <c r="Q21" s="47" t="n">
-        <v>-1.53</v>
+        <v>-1.1</v>
       </c>
       <c r="R21" s="47" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="S21" s="33" t="n">
-        <v>4.23</v>
-      </c>
-      <c r="T21" s="33" t="n">
-        <v>0.17</v>
+        <v>-1.48</v>
+      </c>
+      <c r="S21" s="47" t="n">
+        <v>-4.14</v>
+      </c>
+      <c r="T21" s="47" t="n">
+        <v>-0.02</v>
       </c>
       <c r="U21" s="31" t="inlineStr">
         <is>
@@ -3677,31 +3677,31 @@
         </is>
       </c>
       <c r="C22" s="46" t="n">
-        <v>-0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="D22" s="29" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>8.880000000000001</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F22" s="29" t="n">
-        <v>5.47</v>
+        <v>5.49</v>
       </c>
       <c r="G22" s="29" t="n">
-        <v>4.85</v>
+        <v>4.86</v>
       </c>
       <c r="H22" s="29" t="n">
-        <v>6.45</v>
+        <v>6.46</v>
       </c>
       <c r="I22" s="29" t="n">
-        <v>25.36</v>
+        <v>25.37</v>
       </c>
       <c r="J22" s="29" t="n">
-        <v>70.98</v>
+        <v>71</v>
       </c>
       <c r="K22" s="29" t="n">
-        <v>88.48999999999999</v>
+        <v>88.51000000000001</v>
       </c>
       <c r="L22" s="29" t="n">
         <v>13.84</v>
@@ -3859,17 +3859,17 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>&gt; 7.0</t>
+          <t>&gt; 7.0%</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>3.0 – 7.0</t>
+          <t>3.0% – 7.0%</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>&lt; 3.0</t>
+          <t>&lt; 3.0%</t>
         </is>
       </c>
       <c r="F28" s="27" t="inlineStr">
@@ -3891,17 +3891,17 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>&gt; 0.0</t>
+          <t>&gt; 0.0%</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>-1.0 – 0.0</t>
+          <t>-1.0% – 0.0%</t>
         </is>
       </c>
       <c r="E29" s="31" t="inlineStr">
         <is>
-          <t>&lt; -1.0</t>
+          <t>&lt; -1.0%</t>
         </is>
       </c>
       <c r="F29" s="31" t="inlineStr">
@@ -3923,17 +3923,17 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>&lt; 0.7%</t>
+          <t>&lt; 0.7</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>1.0% – 0.7%</t>
+          <t>1.0 – 0.7</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>&gt; 1.0%</t>
+          <t>&gt; 1.0</t>
         </is>
       </c>
       <c r="F30" s="27" t="inlineStr">
@@ -4137,7 +4137,7 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 10:02 v2.0</t>
+          <t>Generated 2026-05-04 10:06 v2.0</t>
         </is>
       </c>
     </row>
@@ -4232,13 +4232,13 @@
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>14.26530952530278</v>
+        <v>14.26510365921972</v>
       </c>
       <c r="E5" s="29" t="n">
         <v>415.5184553004801</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>59.27499378337036</v>
+        <v>59.27413837180207</v>
       </c>
     </row>
     <row r="6">
@@ -4258,13 +4258,13 @@
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>13.23674325269094</v>
+        <v>13.236552230093</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>91.33928843906948</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>12.09034709951444</v>
+        <v>12.09017262083273</v>
       </c>
     </row>
     <row r="7">
@@ -4284,13 +4284,13 @@
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>8.459328799641117</v>
+        <v>8.459206721050242</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>55.27743647935755</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>4.676100103801618</v>
+        <v>4.676032621886091</v>
       </c>
     </row>
     <row r="8">
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.36969361005393</v>
+        <v>15.36947180634083</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>21.50000333786011</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>3.304484639180467</v>
+        <v>3.304436951374748</v>
       </c>
     </row>
     <row r="9">
@@ -4336,13 +4336,13 @@
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>8.500249996866843</v>
+        <v>8.500127327732415</v>
       </c>
       <c r="E9" s="29" t="n">
         <v>36.52500425066267</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>3.104716672672568</v>
+        <v>3.104671867766003</v>
       </c>
     </row>
     <row r="10">
@@ -4362,13 +4362,13 @@
         </is>
       </c>
       <c r="D10" s="33" t="n">
-        <v>7.040736511754693</v>
+        <v>7.04063490520736</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>43.92423918752959</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>3.092589945986859</v>
+        <v>3.092545316083978</v>
       </c>
     </row>
     <row r="11">
@@ -4388,13 +4388,13 @@
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>7.343034913845621</v>
+        <v>7.34292894475797</v>
       </c>
       <c r="E11" s="29" t="n">
         <v>41.5263607345748</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>3.049295167189306</v>
+        <v>3.049251162083701</v>
       </c>
     </row>
     <row r="12">
@@ -4414,13 +4414,13 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>12.31375315772519</v>
+        <v>12.3150185788605</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>16.58303716504107</v>
+        <v>16.59670043946933</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.041994262556988</v>
+        <v>2.043886742598471</v>
       </c>
     </row>
     <row r="13">
@@ -4440,13 +4440,13 @@
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>7.294415251161368</v>
+        <v>7.294309983715664</v>
       </c>
       <c r="E13" s="29" t="n">
         <v>20.50510328643176</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>1.495727381391869</v>
+        <v>1.495705796193401</v>
       </c>
     </row>
     <row r="14">
@@ -4466,7 +4466,7 @@
         </is>
       </c>
       <c r="D14" s="33" t="n">
-        <v>6.176734980957511</v>
+        <v>6.176645843022274</v>
       </c>
       <c r="E14" s="33" t="n">
         <v>0</v>
@@ -4511,10 +4511,10 @@
         </is>
       </c>
       <c r="B18" s="28" t="n">
-        <v>52442.07356523337</v>
+        <v>52443.24177519698</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>92.42597375466755</v>
+        <v>92.42825096707226</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>6</v>
@@ -4599,10 +4599,10 @@
         </is>
       </c>
       <c r="B25" s="29" t="n">
-        <v>41.77116920492907</v>
+        <v>41.77246629294275</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>19.52938126311098</v>
+        <v>19.5339356879204</v>
       </c>
     </row>
     <row r="26">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>15.5217931241751</v>
+        <v>15.52144736535534</v>
       </c>
       <c r="C26" s="33" t="n">
         <v>29.01250379426139</v>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>10.66269639765878</v>
+        <v>10.66245887862393</v>
       </c>
       <c r="C27" s="29" t="n">
         <v>28.64311527060715</v>
@@ -4638,7 +4638,7 @@
         </is>
       </c>
       <c r="B28" s="33" t="n">
-        <v>24.14476795526446</v>
+        <v>24.14423011363721</v>
       </c>
       <c r="C28" s="33" t="n">
         <v>152.507853974924</v>
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>7.899573317972592</v>
+        <v>7.899397349440786</v>
       </c>
       <c r="C29" s="29" t="n">
         <v>28.64311527060715</v>
@@ -4942,7 +4942,7 @@
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 10:02 v2.0</t>
+          <t>Generated 2026-05-04 10:06 v2.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(optimizer): reword reason and strip green tint from neutral cells
Reason wording:
- The old 'Equities 67.6% → 67%' looked like 'before → after' but was
  actually 'current → target'. That clashed with the new Post-rebal
  column (which is an actual projection). Rewrite reasons in plain
  'at X.X% vs target Y%' form, no arrow.

Cell colors:
- Current %, Target %, and Post-rebal % cells were going through the
  default numeric color picker in _write_data_cell, which paints every
  positive value green. Pass font_color=C['text_pri'] explicitly so
  only the Delta column and the Status pill carry the traffic-light
  semaphore.
- Same fix for Amount (EUR) and % of Portfolio in the Rebalancing
  Actions table.
</commit_message>
<xml_diff>
--- a/output/sample/portfolio_dashboard_sample.xlsx
+++ b/output/sample/portfolio_dashboard_sample.xlsx
@@ -363,7 +363,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -372,7 +372,7 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>80818.52679156253</v>
+        <v>80820.75625323245</v>
       </c>
       <c r="D5" s="2" t="n"/>
     </row>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>26678.52679156253</v>
+        <v>26680.75625323245</v>
       </c>
       <c r="D6" s="2" t="n"/>
     </row>
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>49.27692425482551</v>
+        <v>49.28104221136397</v>
       </c>
       <c r="D7" s="2" t="n"/>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>64.72734237571399</v>
+        <v>64.72831538118703</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>65</v>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>41.78221986945917</v>
+        <v>41.79626795598796</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>55</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>20.61298066766944</v>
+        <v>20.61241205321405</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>25</v>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>24.19739538174008</v>
+        <v>24.19785747467557</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>8</v>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>8.47297670545335</v>
+        <v>8.472742976177967</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>5</v>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="F14" s="22" t="n">
-        <v>15.49538355778712</v>
+        <v>15.50380579197923</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>11</v>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>6.186700251163203</v>
+        <v>6.18652958942094</v>
       </c>
       <c r="C15" s="18" t="n">
         <v>5</v>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="F15" s="17" t="n">
-        <v>9.78236697442971</v>
+        <v>9.766116970263369</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>14</v>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="F16" s="22" t="n">
-        <v>8.742634216583923</v>
+        <v>8.735951807093869</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>12</v>
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="B21" s="28" t="n">
-        <v>12396.80053710938</v>
+        <v>12406.40014648438</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>15.33905779931094</v>
+        <v>15.35051232088437</v>
       </c>
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="12" t="inlineStr">
@@ -1129,7 +1129,7 @@
         <v>11547.61339873075</v>
       </c>
       <c r="C22" s="33" t="n">
-        <v>14.28832454285263</v>
+        <v>14.2879303956883</v>
       </c>
       <c r="D22" s="30" t="n"/>
       <c r="E22" s="34" t="inlineStr">
@@ -1148,7 +1148,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="C23" s="29" t="n">
-        <v>13.25809882704585</v>
+        <v>13.25773309892698</v>
       </c>
       <c r="D23" s="30" t="n"/>
       <c r="E23" s="35" t="inlineStr">
@@ -1167,7 +1167,7 @@
         <v>9961.430530910857</v>
       </c>
       <c r="C24" s="33" t="n">
-        <v>12.3256769535062</v>
+        <v>12.32533694648823</v>
       </c>
       <c r="D24" s="30" t="n"/>
       <c r="E24" s="34" t="inlineStr">
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>6851.339950561523</v>
+        <v>6855.119934082031</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>8.477437318588693</v>
+        <v>8.481880462245561</v>
       </c>
       <c r="D25" s="30" t="n"/>
       <c r="E25" s="12" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:21 v2.0</t>
+          <t>Generated 2026-05-04 13:28 v2.0</t>
         </is>
       </c>
     </row>
@@ -1334,16 +1334,16 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>20.61298066766944</v>
+        <v>20.61241205321405</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>25</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>20.61298066766944</v>
+        <v>20.61241205321405</v>
       </c>
       <c r="E14" s="41" t="n">
-        <v>-4.38701933233056</v>
+        <v>-4.387587946785949</v>
       </c>
       <c r="F14" s="42" t="inlineStr">
         <is>
@@ -1358,16 +1358,16 @@
         </is>
       </c>
       <c r="B15" s="43" t="n">
-        <v>8.47297670545335</v>
+        <v>8.472742976177967</v>
       </c>
       <c r="C15" s="43" t="n">
         <v>5</v>
       </c>
       <c r="D15" s="43" t="n">
-        <v>8.47297670545335</v>
+        <v>8.472742976177967</v>
       </c>
       <c r="E15" s="44" t="n">
-        <v>3.47297670545335</v>
+        <v>3.472742976177967</v>
       </c>
       <c r="F15" s="45" t="inlineStr">
         <is>
@@ -1382,16 +1382,16 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>6.186700251163203</v>
+        <v>6.18652958942094</v>
       </c>
       <c r="C16" s="40" t="n">
         <v>5</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>6.186700251163203</v>
+        <v>6.18652958942094</v>
       </c>
       <c r="E16" s="46" t="n">
-        <v>1.186700251163203</v>
+        <v>1.18652958942094</v>
       </c>
       <c r="F16" s="47" t="inlineStr">
         <is>
@@ -1406,16 +1406,16 @@
         </is>
       </c>
       <c r="B17" s="43" t="n">
-        <v>64.72734237571399</v>
+        <v>64.72831538118703</v>
       </c>
       <c r="C17" s="43" t="n">
         <v>65</v>
       </c>
       <c r="D17" s="43" t="n">
-        <v>64.727342375714</v>
+        <v>64.72831538118703</v>
       </c>
       <c r="E17" s="48" t="n">
-        <v>-0.2726576242859977</v>
+        <v>-0.2716846188129693</v>
       </c>
       <c r="F17" s="49" t="inlineStr">
         <is>
@@ -1493,16 +1493,16 @@
         </is>
       </c>
       <c r="B22" s="40" t="n">
-        <v>24.19739538174008</v>
+        <v>24.19785747467557</v>
       </c>
       <c r="C22" s="40" t="n">
         <v>8</v>
       </c>
       <c r="D22" s="40" t="n">
-        <v>24.19739538174008</v>
+        <v>24.19785747467557</v>
       </c>
       <c r="E22" s="50" t="n">
-        <v>16.19739538174008</v>
+        <v>16.19785747467557</v>
       </c>
       <c r="F22" s="51" t="inlineStr">
         <is>
@@ -1517,16 +1517,16 @@
         </is>
       </c>
       <c r="B23" s="43" t="n">
-        <v>41.78221986945917</v>
+        <v>41.79626795598796</v>
       </c>
       <c r="C23" s="43" t="n">
         <v>55</v>
       </c>
       <c r="D23" s="43" t="n">
-        <v>41.78221986945916</v>
+        <v>41.79626795598796</v>
       </c>
       <c r="E23" s="52" t="n">
-        <v>-13.21778013054084</v>
+        <v>-13.20373204401204</v>
       </c>
       <c r="F23" s="53" t="inlineStr">
         <is>
@@ -1541,16 +1541,16 @@
         </is>
       </c>
       <c r="B24" s="40" t="n">
-        <v>15.49538355778712</v>
+        <v>15.50380579197923</v>
       </c>
       <c r="C24" s="40" t="n">
         <v>11</v>
       </c>
       <c r="D24" s="40" t="n">
-        <v>15.49538355778712</v>
+        <v>15.50380579197923</v>
       </c>
       <c r="E24" s="41" t="n">
-        <v>4.495383557787118</v>
+        <v>4.50380579197923</v>
       </c>
       <c r="F24" s="42" t="inlineStr">
         <is>
@@ -1565,16 +1565,16 @@
         </is>
       </c>
       <c r="B25" s="43" t="n">
-        <v>9.78236697442971</v>
+        <v>9.766116970263369</v>
       </c>
       <c r="C25" s="43" t="n">
         <v>14</v>
       </c>
       <c r="D25" s="43" t="n">
-        <v>9.782366974429706</v>
+        <v>9.766116970263365</v>
       </c>
       <c r="E25" s="44" t="n">
-        <v>-4.217633025570294</v>
+        <v>-4.233883029736635</v>
       </c>
       <c r="F25" s="45" t="inlineStr">
         <is>
@@ -1589,16 +1589,16 @@
         </is>
       </c>
       <c r="B26" s="40" t="n">
-        <v>8.742634216583923</v>
+        <v>8.735951807093869</v>
       </c>
       <c r="C26" s="40" t="n">
         <v>12</v>
       </c>
       <c r="D26" s="40" t="n">
-        <v>8.742634216583921</v>
+        <v>8.735951807093867</v>
       </c>
       <c r="E26" s="41" t="n">
-        <v>-3.257365783416079</v>
+        <v>-3.264048192906133</v>
       </c>
       <c r="F26" s="42" t="inlineStr">
         <is>
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="B30" s="40" t="n">
-        <v>22.07463495089159</v>
+        <v>22.07369419634397</v>
       </c>
       <c r="C30" s="40" t="n">
         <v>10</v>
       </c>
       <c r="D30" s="40" t="n">
-        <v>22.07463495089159</v>
+        <v>22.07369419634397</v>
       </c>
       <c r="E30" s="50" t="n">
-        <v>12.07463495089159</v>
+        <v>12.07369419634397</v>
       </c>
       <c r="F30" s="51" t="inlineStr">
         <is>
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="B31" s="43" t="n">
-        <v>10.83887863662915</v>
+        <v>10.81089082353887</v>
       </c>
       <c r="C31" s="43" t="n">
         <v>15</v>
       </c>
       <c r="D31" s="43" t="n">
-        <v>10.83887863662915</v>
+        <v>10.81089082353887</v>
       </c>
       <c r="E31" s="44" t="n">
-        <v>-4.161121363370849</v>
+        <v>-4.189109176461129</v>
       </c>
       <c r="F31" s="45" t="inlineStr">
         <is>
@@ -1700,16 +1700,16 @@
         </is>
       </c>
       <c r="B32" s="40" t="n">
-        <v>11.24892110411809</v>
+        <v>11.25465370943649</v>
       </c>
       <c r="C32" s="40" t="n">
         <v>15</v>
       </c>
       <c r="D32" s="40" t="n">
-        <v>11.24892110411809</v>
+        <v>11.25465370943649</v>
       </c>
       <c r="E32" s="41" t="n">
-        <v>-3.751078895881914</v>
+        <v>-3.745346290563509</v>
       </c>
       <c r="F32" s="42" t="inlineStr">
         <is>
@@ -1724,16 +1724,16 @@
         </is>
       </c>
       <c r="B33" s="43" t="n">
-        <v>13.09715030377868</v>
+        <v>13.10381772226808</v>
       </c>
       <c r="C33" s="43" t="n">
         <v>15</v>
       </c>
       <c r="D33" s="43" t="n">
-        <v>13.09715030377868</v>
+        <v>13.10381772226808</v>
       </c>
       <c r="E33" s="48" t="n">
-        <v>-1.902849696221319</v>
+        <v>-1.896182277731922</v>
       </c>
       <c r="F33" s="49" t="inlineStr">
         <is>
@@ -1748,16 +1748,16 @@
         </is>
       </c>
       <c r="B34" s="40" t="n">
-        <v>23.69795705541933</v>
+        <v>23.71529713153314</v>
       </c>
       <c r="C34" s="40" t="n">
         <v>25</v>
       </c>
       <c r="D34" s="40" t="n">
-        <v>23.69795705541933</v>
+        <v>23.71529713153314</v>
       </c>
       <c r="E34" s="46" t="n">
-        <v>-1.30204294458067</v>
+        <v>-1.284702868466862</v>
       </c>
       <c r="F34" s="47" t="inlineStr">
         <is>
@@ -1772,16 +1772,16 @@
         </is>
       </c>
       <c r="B35" s="43" t="n">
-        <v>19.04245794916315</v>
+        <v>19.04164641687945</v>
       </c>
       <c r="C35" s="43" t="n">
         <v>20</v>
       </c>
       <c r="D35" s="43" t="n">
-        <v>19.04245794916315</v>
+        <v>19.04164641687945</v>
       </c>
       <c r="E35" s="48" t="n">
-        <v>-0.957542050836846</v>
+        <v>-0.9583535831205516</v>
       </c>
       <c r="F35" s="49" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
     <row r="53">
       <c r="A53" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:21 v2.0</t>
+          <t>Generated 2026-05-04 13:28 v2.0</t>
         </is>
       </c>
     </row>
@@ -2204,25 +2204,25 @@
         <v>128</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>154.9600067138672</v>
+        <v>155.0800018310547</v>
       </c>
       <c r="J4" s="28" t="n">
         <v>10240</v>
       </c>
       <c r="K4" s="28" t="n">
-        <v>12396.80053710938</v>
+        <v>12406.40014648438</v>
       </c>
       <c r="L4" s="29" t="n">
-        <v>15.33905779931094</v>
+        <v>15.35051232088437</v>
       </c>
       <c r="M4" s="29" t="n">
-        <v>23.69795705541933</v>
+        <v>23.71529713153314</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>2156.800537109375</v>
+        <v>2166.400146484375</v>
       </c>
       <c r="O4" s="29" t="n">
-        <v>21.06250524520874</v>
+        <v>21.15625143051147</v>
       </c>
       <c r="P4" s="27" t="inlineStr">
         <is>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="S4" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2292,10 +2292,10 @@
         <v>11547.61339873075</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>14.28832454285263</v>
+        <v>14.2879303956883</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>22.07463495089159</v>
+        <v>22.07369419634397</v>
       </c>
       <c r="N5" s="32" t="n">
         <v>9307.613398730755</v>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="S5" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2371,10 +2371,10 @@
         <v>9961.430530910857</v>
       </c>
       <c r="L6" s="29" t="n">
-        <v>12.3256769535062</v>
+        <v>12.32533694648823</v>
       </c>
       <c r="M6" s="29" t="n">
-        <v>19.04245794916315</v>
+        <v>19.04164641687945</v>
       </c>
       <c r="N6" s="28" t="n">
         <v>1411.430530910857</v>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2441,25 +2441,25 @@
         <v>56</v>
       </c>
       <c r="I7" s="32" t="n">
-        <v>76.12599945068359</v>
+        <v>76.16799926757812</v>
       </c>
       <c r="J7" s="32" t="n">
         <v>5040</v>
       </c>
       <c r="K7" s="32" t="n">
-        <v>6851.339950561523</v>
+        <v>6855.119934082031</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>8.477437318588693</v>
+        <v>8.481880462245561</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>13.09715030377868</v>
+        <v>13.10381772226808</v>
       </c>
       <c r="N7" s="32" t="n">
-        <v>1811.339950561523</v>
+        <v>1815.119934082031</v>
       </c>
       <c r="O7" s="33" t="n">
-        <v>35.93928473336356</v>
+        <v>36.01428440638951</v>
       </c>
       <c r="P7" s="31" t="inlineStr">
         <is>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="S7" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2520,25 +2520,25 @@
         <v>98</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>117.6900024414062</v>
+        <v>117.754997253418</v>
       </c>
       <c r="J8" s="28" t="n">
         <v>4900</v>
       </c>
       <c r="K8" s="28" t="n">
-        <v>5884.500122070312</v>
+        <v>5887.749862670898</v>
       </c>
       <c r="L8" s="29" t="n">
-        <v>7.28112767663646</v>
+        <v>7.284947748104517</v>
       </c>
       <c r="M8" s="29" t="n">
-        <v>11.24892110411809</v>
+        <v>11.25465370943649</v>
       </c>
       <c r="N8" s="28" t="n">
-        <v>984.5001220703125</v>
+        <v>987.7498626708984</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>20.09183922592474</v>
+        <v>20.1581604626714</v>
       </c>
       <c r="P8" s="27" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="S8" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2599,25 +2599,25 @@
         <v>33</v>
       </c>
       <c r="I9" s="32" t="n">
-        <v>47.25</v>
+        <v>47.13000106811523</v>
       </c>
       <c r="J9" s="32" t="n">
         <v>3960</v>
       </c>
       <c r="K9" s="32" t="n">
-        <v>5670</v>
+        <v>5655.600128173828</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v>7.015718084819072</v>
+        <v>6.997707507776049</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v>10.83887863662915</v>
+        <v>10.81089082353887</v>
       </c>
       <c r="N9" s="32" t="n">
-        <v>1710</v>
+        <v>1695.600128173828</v>
       </c>
       <c r="O9" s="33" t="n">
-        <v>43.18181818181818</v>
+        <v>42.81818505489465</v>
       </c>
       <c r="P9" s="31" t="inlineStr">
         <is>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="S9" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="L10" s="29" t="n">
-        <v>13.25809882704585</v>
+        <v>13.25773309892698</v>
       </c>
       <c r="M10" s="29" t="n">
         <v>64.31917363528412</v>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="S10" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
         <v>5944.107150852142</v>
       </c>
       <c r="L11" s="33" t="n">
-        <v>7.354881840623588</v>
+        <v>7.354678954287075</v>
       </c>
       <c r="M11" s="33" t="n">
         <v>35.68082636471589</v>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="S11" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
         <v>5000</v>
       </c>
       <c r="L12" s="29" t="n">
-        <v>6.186700251163203</v>
+        <v>6.18652958942094</v>
       </c>
       <c r="M12" s="29" t="n">
         <v>100</v>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="S12" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
         <v>6847.734948739668</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v>8.47297670545335</v>
+        <v>8.472742976177967</v>
       </c>
       <c r="M13" s="33" t="n">
         <v>100</v>
@@ -2952,14 +2952,14 @@
       </c>
       <c r="S13" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:21</t>
+          <t>2026-05-04 13:28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:21 v2.0</t>
+          <t>Generated 2026-05-04 13:28 v2.0</t>
         </is>
       </c>
     </row>
@@ -3149,13 +3149,13 @@
         <v>6.58</v>
       </c>
       <c r="H5" s="60" t="n">
-        <v>6.98</v>
+        <v>6.99</v>
       </c>
       <c r="I5" s="60" t="n">
         <v>22</v>
       </c>
       <c r="J5" s="60" t="n">
-        <v>48.91</v>
+        <v>48.92</v>
       </c>
       <c r="K5" s="60" t="n">
         <v>45.09</v>
@@ -3276,31 +3276,31 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>6.64</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>4.47</v>
+        <v>4.46</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>6.39</v>
+        <v>6.38</v>
       </c>
       <c r="H7" s="33" t="n">
         <v>6.52</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>23.69</v>
+        <v>23.68</v>
       </c>
       <c r="J7" s="33" t="n">
         <v>56.16</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>58.74</v>
+        <v>58.73</v>
       </c>
       <c r="L7" s="33" t="n">
         <v>9.83</v>
@@ -3495,25 +3495,25 @@
         <v>0.59</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>5.97</v>
+        <v>5.96</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>3.98</v>
+        <v>3.97</v>
       </c>
       <c r="G10" s="29" t="n">
         <v>5.08</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>5.37</v>
+        <v>5.36</v>
       </c>
       <c r="I10" s="29" t="n">
         <v>21.74</v>
       </c>
       <c r="J10" s="29" t="n">
-        <v>55.7</v>
+        <v>55.69</v>
       </c>
       <c r="K10" s="29" t="n">
-        <v>63.3</v>
+        <v>63.29</v>
       </c>
       <c r="L10" s="29" t="n">
         <v>10.47</v>
@@ -3906,7 +3906,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
@@ -3915,58 +3915,58 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.91</v>
+        <v>1.03</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>7.26</v>
+        <v>7.75</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>4.18</v>
+        <v>4.71</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>5.33</v>
+        <v>6.61</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>5.72</v>
+        <v>6.85</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>22.87</v>
+        <v>24.62</v>
       </c>
       <c r="J16" s="29" t="n">
-        <v>62.56</v>
+        <v>62.81</v>
       </c>
       <c r="K16" s="29" t="n">
-        <v>75.01000000000001</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="L16" s="29" t="n">
-        <v>12.15</v>
+        <v>11.52</v>
       </c>
       <c r="M16" s="29" t="n">
-        <v>14.24</v>
+        <v>13.8</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="P16" s="62" t="n">
-        <v>-21.73</v>
+        <v>-21.07</v>
       </c>
       <c r="Q16" s="62" t="n">
-        <v>-1.45</v>
+        <v>-1.39</v>
       </c>
       <c r="R16" s="62" t="n">
-        <v>-2.19</v>
+        <v>-2.13</v>
       </c>
       <c r="S16" s="29" t="n">
-        <v>6.34</v>
+        <v>5.92</v>
       </c>
       <c r="T16" s="29" t="n">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="U16" s="27" t="inlineStr">
         <is>
@@ -3977,7 +3977,7 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B17" s="31" t="inlineStr">
@@ -3986,58 +3986,58 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>0.65</v>
+        <v>0.62</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>7.67</v>
+        <v>7.32</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>4.63</v>
+        <v>4.24</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>6.53</v>
+        <v>5.39</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>6.77</v>
+        <v>5.78</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>24.53</v>
+        <v>22.94</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>62.69</v>
+        <v>62.65</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>70.15000000000001</v>
+        <v>75.11</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v>11.51</v>
+        <v>12.16</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>13.8</v>
+        <v>14.24</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>0.54</v>
+        <v>0.57</v>
       </c>
       <c r="O17" s="33" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="P17" s="63" t="n">
-        <v>-21.07</v>
+        <v>-21.73</v>
       </c>
       <c r="Q17" s="63" t="n">
-        <v>-1.39</v>
+        <v>-1.45</v>
       </c>
       <c r="R17" s="63" t="n">
-        <v>-2.13</v>
+        <v>-2.19</v>
       </c>
       <c r="S17" s="33" t="n">
-        <v>5.9</v>
+        <v>6.35</v>
       </c>
       <c r="T17" s="33" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="U17" s="31" t="inlineStr">
         <is>
@@ -4057,34 +4057,34 @@
         </is>
       </c>
       <c r="C18" s="29" t="n">
-        <v>1.78</v>
+        <v>1.83</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>1.36</v>
+        <v>1.42</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>12.54</v>
+        <v>12.6</v>
       </c>
       <c r="F18" s="29" t="n">
-        <v>8.84</v>
+        <v>8.9</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>16.45</v>
+        <v>16.52</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>16.06</v>
+        <v>16.12</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>40.65</v>
+        <v>40.72</v>
       </c>
       <c r="J18" s="29" t="n">
-        <v>68.56</v>
+        <v>68.66</v>
       </c>
       <c r="K18" s="29" t="n">
-        <v>42.04</v>
+        <v>42.12</v>
       </c>
       <c r="L18" s="29" t="n">
-        <v>7.55</v>
+        <v>7.56</v>
       </c>
       <c r="M18" s="29" t="n">
         <v>18.82</v>
@@ -4105,7 +4105,7 @@
         <v>-2.59</v>
       </c>
       <c r="S18" s="29" t="n">
-        <v>2.73</v>
+        <v>2.74</v>
       </c>
       <c r="T18" s="29" t="n">
         <v>0.1</v>
@@ -4412,43 +4412,43 @@
         </is>
       </c>
       <c r="C23" s="63" t="n">
-        <v>-0.31</v>
-      </c>
-      <c r="D23" s="33" t="n">
-        <v>0.15</v>
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="D23" s="63" t="n">
+        <v>-0.11</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>4.35</v>
+        <v>4.09</v>
       </c>
       <c r="F23" s="63" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-1.19</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>7.24</v>
+        <v>6.97</v>
       </c>
       <c r="H23" s="33" t="n">
-        <v>2.3</v>
+        <v>2.04</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>14.57</v>
+        <v>14.28</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>40.38</v>
+        <v>40.02</v>
       </c>
       <c r="K23" s="33" t="n">
-        <v>54.73</v>
+        <v>54.34</v>
       </c>
       <c r="L23" s="33" t="n">
-        <v>9.539999999999999</v>
+        <v>9.48</v>
       </c>
       <c r="M23" s="33" t="n">
-        <v>14.94</v>
+        <v>14.95</v>
       </c>
       <c r="N23" s="33" t="n">
         <v>0.37</v>
       </c>
       <c r="O23" s="33" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="P23" s="63" t="n">
         <v>-22.86</v>
@@ -4460,7 +4460,7 @@
         <v>-2.22</v>
       </c>
       <c r="S23" s="33" t="n">
-        <v>4.11</v>
+        <v>4.06</v>
       </c>
       <c r="T23" s="33" t="n">
         <v>0.17</v>
@@ -4801,7 +4801,7 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:21 v2.0</t>
+          <t>Generated 2026-05-04 13:28 v2.0</t>
         </is>
       </c>
     </row>
@@ -4896,13 +4896,13 @@
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>14.28832454285263</v>
+        <v>14.2879303956883</v>
       </c>
       <c r="E5" s="29" t="n">
         <v>415.5184553004801</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>59.37062542878062</v>
+        <v>59.36898767457182</v>
       </c>
     </row>
     <row r="6">
@@ -4922,13 +4922,13 @@
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>13.25809882704585</v>
+        <v>13.25773309892698</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>91.33928843906948</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>12.1098531291723</v>
+        <v>12.10951907571089</v>
       </c>
     </row>
     <row r="7">
@@ -4948,13 +4948,13 @@
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>8.47297670545335</v>
+        <v>8.472742976177967</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>55.27743647935755</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>4.683644316267737</v>
+        <v>4.683515116716004</v>
       </c>
     </row>
     <row r="8">
@@ -4974,65 +4974,65 @@
         </is>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.33905779931094</v>
+        <v>15.35051232088437</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>21.06250524520874</v>
+        <v>21.15625143051147</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>3.230789853545467</v>
+        <v>3.24759298247794</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
+          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>IE00B1FZS798</t>
+          <t>LU0292107645</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>IBTM.L</t>
+          <t>XMME.DE</t>
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>7.354881840623588</v>
+        <v>8.481880462245561</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>41.5263607345748</v>
+        <v>36.01428440638951</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>3.054214764739086</v>
+        <v>3.054688552683102</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
+          <t>iShares $ Treasury Bond 7-10yr UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>LU0292107645</t>
+          <t>IE00B1FZS798</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
-          <t>XMME.DE</t>
+          <t>IBTM.L</t>
         </is>
       </c>
       <c r="D10" s="33" t="n">
-        <v>8.477437318588693</v>
+        <v>7.354678954287075</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>35.93928473336356</v>
+        <v>41.5263607345748</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>3.046730336020011</v>
+        <v>3.054130513427105</v>
       </c>
     </row>
     <row r="11">
@@ -5052,13 +5052,13 @@
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>7.015718084819072</v>
+        <v>6.997707507776049</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>43.18181818181818</v>
+        <v>42.81818505489465</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>3.029514627535509</v>
+        <v>2.996291350279805</v>
       </c>
     </row>
     <row r="12">
@@ -5078,13 +5078,13 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>12.3256769535062</v>
+        <v>12.32533694648823</v>
       </c>
       <c r="E12" s="33" t="n">
         <v>16.50795942585797</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.03471775044713</v>
+        <v>2.034661622226559</v>
       </c>
     </row>
     <row r="13">
@@ -5104,13 +5104,13 @@
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>7.28112767663646</v>
+        <v>7.284947748104517</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>20.09183922592474</v>
+        <v>20.1581604626714</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>1.462912466624107</v>
+        <v>1.468511456684675</v>
       </c>
     </row>
     <row r="14">
@@ -5130,7 +5130,7 @@
         </is>
       </c>
       <c r="D14" s="33" t="n">
-        <v>6.186700251163203</v>
+        <v>6.18652958942094</v>
       </c>
       <c r="E14" s="33" t="n">
         <v>0</v>
@@ -5175,10 +5175,10 @@
         </is>
       </c>
       <c r="B18" s="28" t="n">
-        <v>52311.68453938283</v>
+        <v>52313.91400105275</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>92.05031035210889</v>
+        <v>92.02888268013419</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>6</v>
@@ -5263,10 +5263,10 @@
         </is>
       </c>
       <c r="B25" s="29" t="n">
-        <v>41.78221986945917</v>
+        <v>41.79626795598796</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>19.22076796566382</v>
+        <v>19.27412377301361</v>
       </c>
     </row>
     <row r="26">
@@ -5276,10 +5276,10 @@
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>15.49538355778712</v>
+        <v>15.50380579197923</v>
       </c>
       <c r="C26" s="33" t="n">
-        <v>28.50089498928615</v>
+        <v>28.58526791845049</v>
       </c>
     </row>
     <row r="27">
@@ -5289,10 +5289,10 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>9.78236697442971</v>
+        <v>9.766116970263369</v>
       </c>
       <c r="C27" s="29" t="n">
-        <v>28.11205421765055</v>
+        <v>28.04419898269251</v>
       </c>
     </row>
     <row r="28">
@@ -5302,10 +5302,10 @@
         </is>
       </c>
       <c r="B28" s="33" t="n">
-        <v>24.19739538174008</v>
+        <v>24.19785747467557</v>
       </c>
       <c r="C28" s="33" t="n">
-        <v>152.2242665905379</v>
+        <v>152.2776223978877</v>
       </c>
     </row>
     <row r="29">
@@ -5315,10 +5315,10 @@
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>8.742634216583923</v>
+        <v>8.735951807093869</v>
       </c>
       <c r="C29" s="29" t="n">
-        <v>28.11205421765055</v>
+        <v>28.04419898269251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
style(excel): drop inline units from data cells, carry them in headers
Follow the convention: units belong in the column / label name, data
cells show bare numbers. Applied consistently across the workbook:

Hero KPIs (Dashboard):
- 'Total Value (AuM)' → 'Total Value (EUR)', number only (no € in cell)
- 'Total Gain' → 'Total Gain (EUR)', signed number only
- 'RTD (Return to Date)' → 'RTD (%)', signed number only

Optimizer:
- Allocation deviations: Current %, Target %, Post-rebal % cells use
  plain 0.00 format (header already names the unit)
- Delta after rebal (pp) uses signed format without %
- Rebalancing actions: Amount (EUR) and % of Portfolio cells are plain
  numbers

All 51 tests still pass and the sample dashboard regenerates cleanly.
</commit_message>
<xml_diff>
--- a/output/sample/portfolio_dashboard_sample.xlsx
+++ b/output/sample/portfolio_dashboard_sample.xlsx
@@ -20,11 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="&quot;€&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="&quot;€&quot;+#,##0.00;&quot;€&quot;-#,##0.00;&quot;€&quot;0.00"/>
-    <numFmt numFmtId="166" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;;0.00&quot;%&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.00&quot;%&quot;"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="+#,##0.00;-#,##0.00;0.00"/>
+    <numFmt numFmtId="165" formatCode="+0.00;-0.00;0.00"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -254,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -268,16 +266,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -363,43 +361,37 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -860,33 +852,33 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Total Value (AuM)</t>
+          <t>Total Value (EUR)</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>80820.75625323245</v>
+        <v>80831.37868844786</v>
       </c>
       <c r="D5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Total Gain</t>
+          <t>Total Gain (EUR)</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>26680.75625323245</v>
+        <v>26691.37868844786</v>
       </c>
       <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>RTD (Return to Date)</t>
+          <t>RTD (%)</t>
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>49.28104221136397</v>
+        <v>49.30066252022139</v>
       </c>
       <c r="D7" s="2" t="n"/>
     </row>
@@ -950,7 +942,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>64.72831538118703</v>
+        <v>64.73295060071293</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>65</v>
@@ -962,7 +954,7 @@
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>41.79626795598796</v>
+        <v>41.79516167143485</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>55</v>
@@ -975,7 +967,7 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>20.61241205321405</v>
+        <v>20.60970327828998</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>25</v>
@@ -987,7 +979,7 @@
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>24.19785747467557</v>
+        <v>24.19321790615446</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>8</v>
@@ -1000,7 +992,7 @@
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>8.472742976177967</v>
+        <v>8.471629532799646</v>
       </c>
       <c r="C14" s="14" t="n">
         <v>5</v>
@@ -1012,7 +1004,7 @@
         </is>
       </c>
       <c r="F14" s="22" t="n">
-        <v>15.50380579197923</v>
+        <v>15.50544013183685</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>11</v>
@@ -1025,7 +1017,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>6.18652958942094</v>
+        <v>6.185716588197428</v>
       </c>
       <c r="C15" s="18" t="n">
         <v>5</v>
@@ -1037,7 +1029,7 @@
         </is>
       </c>
       <c r="F15" s="17" t="n">
-        <v>9.766116970263369</v>
+        <v>9.768936068831742</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>14</v>
@@ -1051,7 +1043,7 @@
         </is>
       </c>
       <c r="F16" s="22" t="n">
-        <v>8.735951807093869</v>
+        <v>8.737244221742097</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>12</v>
@@ -1107,10 +1099,10 @@
         </is>
       </c>
       <c r="B21" s="28" t="n">
-        <v>12406.40014648438</v>
+        <v>12408.00048828125</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>15.35051232088437</v>
+        <v>15.35047488934462</v>
       </c>
       <c r="D21" s="30" t="n"/>
       <c r="E21" s="12" t="inlineStr">
@@ -1129,7 +1121,7 @@
         <v>11547.61339873075</v>
       </c>
       <c r="C22" s="33" t="n">
-        <v>14.2879303956883</v>
+        <v>14.28605275092394</v>
       </c>
       <c r="D22" s="30" t="n"/>
       <c r="E22" s="34" t="inlineStr">
@@ -1148,7 +1140,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="C23" s="29" t="n">
-        <v>13.25773309892698</v>
+        <v>13.25599083728018</v>
       </c>
       <c r="D23" s="30" t="n"/>
       <c r="E23" s="35" t="inlineStr">
@@ -1164,10 +1156,10 @@
         </is>
       </c>
       <c r="B24" s="32" t="n">
-        <v>9961.430530910857</v>
+        <v>9963.762713440719</v>
       </c>
       <c r="C24" s="33" t="n">
-        <v>12.32533694648823</v>
+        <v>12.32660245947866</v>
       </c>
       <c r="D24" s="30" t="n"/>
       <c r="E24" s="34" t="inlineStr">
@@ -1183,10 +1175,10 @@
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>6855.119934082031</v>
+        <v>6857.460021972656</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>8.481880462245561</v>
+        <v>8.483660842163392</v>
       </c>
       <c r="D25" s="30" t="n"/>
       <c r="E25" s="12" t="inlineStr">
@@ -1201,7 +1193,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:28 v2.0</t>
+          <t>Generated 2026-05-04 13:36 v2.0</t>
         </is>
       </c>
     </row>
@@ -1333,19 +1325,19 @@
           <t>Fixed Income</t>
         </is>
       </c>
-      <c r="B14" s="40" t="n">
-        <v>20.61241205321405</v>
-      </c>
-      <c r="C14" s="40" t="n">
+      <c r="B14" s="14" t="n">
+        <v>20.60970327828998</v>
+      </c>
+      <c r="C14" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="40" t="n">
-        <v>20.61241205321405</v>
-      </c>
-      <c r="E14" s="41" t="n">
-        <v>-4.387587946785949</v>
-      </c>
-      <c r="F14" s="42" t="inlineStr">
+      <c r="D14" s="14" t="n">
+        <v>20.60970327828998</v>
+      </c>
+      <c r="E14" s="40" t="n">
+        <v>-4.390296721710016</v>
+      </c>
+      <c r="F14" s="41" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1357,19 +1349,19 @@
           <t>Commodities</t>
         </is>
       </c>
-      <c r="B15" s="43" t="n">
-        <v>8.472742976177967</v>
-      </c>
-      <c r="C15" s="43" t="n">
+      <c r="B15" s="18" t="n">
+        <v>8.471629532799646</v>
+      </c>
+      <c r="C15" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="43" t="n">
-        <v>8.472742976177967</v>
-      </c>
-      <c r="E15" s="44" t="n">
-        <v>3.472742976177967</v>
-      </c>
-      <c r="F15" s="45" t="inlineStr">
+      <c r="D15" s="18" t="n">
+        <v>8.471629532799646</v>
+      </c>
+      <c r="E15" s="42" t="n">
+        <v>3.471629532799646</v>
+      </c>
+      <c r="F15" s="43" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1381,19 +1373,19 @@
           <t>Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="B16" s="40" t="n">
-        <v>6.18652958942094</v>
-      </c>
-      <c r="C16" s="40" t="n">
+      <c r="B16" s="14" t="n">
+        <v>6.185716588197428</v>
+      </c>
+      <c r="C16" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D16" s="40" t="n">
-        <v>6.18652958942094</v>
-      </c>
-      <c r="E16" s="46" t="n">
-        <v>1.18652958942094</v>
-      </c>
-      <c r="F16" s="47" t="inlineStr">
+      <c r="D16" s="14" t="n">
+        <v>6.185716588197428</v>
+      </c>
+      <c r="E16" s="44" t="n">
+        <v>1.185716588197428</v>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1405,19 +1397,19 @@
           <t>Equities</t>
         </is>
       </c>
-      <c r="B17" s="43" t="n">
-        <v>64.72831538118703</v>
-      </c>
-      <c r="C17" s="43" t="n">
+      <c r="B17" s="18" t="n">
+        <v>64.73295060071293</v>
+      </c>
+      <c r="C17" s="18" t="n">
         <v>65</v>
       </c>
-      <c r="D17" s="43" t="n">
-        <v>64.72831538118703</v>
-      </c>
-      <c r="E17" s="48" t="n">
-        <v>-0.2716846188129693</v>
-      </c>
-      <c r="F17" s="49" t="inlineStr">
+      <c r="D17" s="18" t="n">
+        <v>64.73295060071294</v>
+      </c>
+      <c r="E17" s="46" t="n">
+        <v>-0.2670493992870604</v>
+      </c>
+      <c r="F17" s="47" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1429,19 +1421,19 @@
           <t>Alternative</t>
         </is>
       </c>
-      <c r="B18" s="40" t="n">
+      <c r="B18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="40" t="n">
+      <c r="C18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="40" t="n">
+      <c r="D18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="46" t="n">
+      <c r="E18" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="47" t="inlineStr">
+      <c r="F18" s="45" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1492,19 +1484,19 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="B22" s="40" t="n">
-        <v>24.19785747467557</v>
-      </c>
-      <c r="C22" s="40" t="n">
+      <c r="B22" s="14" t="n">
+        <v>24.19321790615446</v>
+      </c>
+      <c r="C22" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="40" t="n">
-        <v>24.19785747467557</v>
-      </c>
-      <c r="E22" s="50" t="n">
-        <v>16.19785747467557</v>
-      </c>
-      <c r="F22" s="51" t="inlineStr">
+      <c r="D22" s="14" t="n">
+        <v>24.19321790615446</v>
+      </c>
+      <c r="E22" s="48" t="n">
+        <v>16.19321790615446</v>
+      </c>
+      <c r="F22" s="49" t="inlineStr">
         <is>
           <t>● Action</t>
         </is>
@@ -1516,19 +1508,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B23" s="43" t="n">
-        <v>41.79626795598796</v>
-      </c>
-      <c r="C23" s="43" t="n">
+      <c r="B23" s="18" t="n">
+        <v>41.79516167143485</v>
+      </c>
+      <c r="C23" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="D23" s="43" t="n">
-        <v>41.79626795598796</v>
-      </c>
-      <c r="E23" s="52" t="n">
-        <v>-13.20373204401204</v>
-      </c>
-      <c r="F23" s="53" t="inlineStr">
+      <c r="D23" s="18" t="n">
+        <v>41.79516167143485</v>
+      </c>
+      <c r="E23" s="50" t="n">
+        <v>-13.20483832856515</v>
+      </c>
+      <c r="F23" s="51" t="inlineStr">
         <is>
           <t>● Action</t>
         </is>
@@ -1540,19 +1532,19 @@
           <t>Emerging Markets</t>
         </is>
       </c>
-      <c r="B24" s="40" t="n">
-        <v>15.50380579197923</v>
-      </c>
-      <c r="C24" s="40" t="n">
+      <c r="B24" s="14" t="n">
+        <v>15.50544013183685</v>
+      </c>
+      <c r="C24" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="D24" s="40" t="n">
-        <v>15.50380579197923</v>
-      </c>
-      <c r="E24" s="41" t="n">
-        <v>4.50380579197923</v>
-      </c>
-      <c r="F24" s="42" t="inlineStr">
+      <c r="D24" s="14" t="n">
+        <v>15.50544013183685</v>
+      </c>
+      <c r="E24" s="40" t="n">
+        <v>4.505440131836851</v>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1564,19 +1556,19 @@
           <t>Eurozone EMU</t>
         </is>
       </c>
-      <c r="B25" s="43" t="n">
-        <v>9.766116970263369</v>
-      </c>
-      <c r="C25" s="43" t="n">
+      <c r="B25" s="18" t="n">
+        <v>9.768936068831742</v>
+      </c>
+      <c r="C25" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="D25" s="43" t="n">
-        <v>9.766116970263365</v>
-      </c>
-      <c r="E25" s="44" t="n">
-        <v>-4.233883029736635</v>
-      </c>
-      <c r="F25" s="45" t="inlineStr">
+      <c r="D25" s="18" t="n">
+        <v>9.76893606883174</v>
+      </c>
+      <c r="E25" s="42" t="n">
+        <v>-4.23106393116826</v>
+      </c>
+      <c r="F25" s="43" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1588,19 +1580,19 @@
           <t>Dev ex-USA ex-EMU ex-JP</t>
         </is>
       </c>
-      <c r="B26" s="40" t="n">
-        <v>8.735951807093869</v>
-      </c>
-      <c r="C26" s="40" t="n">
+      <c r="B26" s="14" t="n">
+        <v>8.737244221742097</v>
+      </c>
+      <c r="C26" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D26" s="40" t="n">
-        <v>8.735951807093867</v>
-      </c>
-      <c r="E26" s="41" t="n">
-        <v>-3.264048192906133</v>
-      </c>
-      <c r="F26" s="42" t="inlineStr">
+      <c r="D26" s="14" t="n">
+        <v>8.737244221742097</v>
+      </c>
+      <c r="E26" s="40" t="n">
+        <v>-3.262755778257903</v>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1651,19 +1643,19 @@
           <t>CNKY.L</t>
         </is>
       </c>
-      <c r="B30" s="40" t="n">
-        <v>22.07369419634397</v>
-      </c>
-      <c r="C30" s="40" t="n">
+      <c r="B30" s="14" t="n">
+        <v>22.06921300257647</v>
+      </c>
+      <c r="C30" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="40" t="n">
-        <v>22.07369419634397</v>
-      </c>
-      <c r="E30" s="50" t="n">
-        <v>12.07369419634397</v>
-      </c>
-      <c r="F30" s="51" t="inlineStr">
+      <c r="D30" s="14" t="n">
+        <v>22.06921300257647</v>
+      </c>
+      <c r="E30" s="48" t="n">
+        <v>12.06921300257647</v>
+      </c>
+      <c r="F30" s="49" t="inlineStr">
         <is>
           <t>● Action</t>
         </is>
@@ -1675,19 +1667,19 @@
           <t>VERX.DE</t>
         </is>
       </c>
-      <c r="B31" s="43" t="n">
-        <v>10.81089082353887</v>
-      </c>
-      <c r="C31" s="43" t="n">
+      <c r="B31" s="18" t="n">
+        <v>10.81557595561772</v>
+      </c>
+      <c r="C31" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="D31" s="43" t="n">
-        <v>10.81089082353887</v>
-      </c>
-      <c r="E31" s="44" t="n">
-        <v>-4.189109176461129</v>
-      </c>
-      <c r="F31" s="45" t="inlineStr">
+      <c r="D31" s="18" t="n">
+        <v>10.81557595561772</v>
+      </c>
+      <c r="E31" s="42" t="n">
+        <v>-4.184424044382277</v>
+      </c>
+      <c r="F31" s="43" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1699,19 +1691,19 @@
           <t>EUNL.DE</t>
         </is>
       </c>
-      <c r="B32" s="40" t="n">
-        <v>11.25465370943649</v>
-      </c>
-      <c r="C32" s="40" t="n">
+      <c r="B32" s="14" t="n">
+        <v>11.25380219913764</v>
+      </c>
+      <c r="C32" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D32" s="40" t="n">
-        <v>11.25465370943649</v>
-      </c>
-      <c r="E32" s="41" t="n">
-        <v>-3.745346290563509</v>
-      </c>
-      <c r="F32" s="42" t="inlineStr">
+      <c r="D32" s="14" t="n">
+        <v>11.25380219913764</v>
+      </c>
+      <c r="E32" s="40" t="n">
+        <v>-3.746197800862364</v>
+      </c>
+      <c r="F32" s="41" t="inlineStr">
         <is>
           <t>● Drift</t>
         </is>
@@ -1723,19 +1715,19 @@
           <t>XMME.DE</t>
         </is>
       </c>
-      <c r="B33" s="43" t="n">
-        <v>13.10381772226808</v>
-      </c>
-      <c r="C33" s="43" t="n">
+      <c r="B33" s="18" t="n">
+        <v>13.10562976573164</v>
+      </c>
+      <c r="C33" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="D33" s="43" t="n">
-        <v>13.10381772226808</v>
-      </c>
-      <c r="E33" s="48" t="n">
-        <v>-1.896182277731922</v>
-      </c>
-      <c r="F33" s="49" t="inlineStr">
+      <c r="D33" s="18" t="n">
+        <v>13.10562976573164</v>
+      </c>
+      <c r="E33" s="46" t="n">
+        <v>-1.894370234268361</v>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1747,19 +1739,19 @@
           <t>VWCE.DE</t>
         </is>
       </c>
-      <c r="B34" s="40" t="n">
-        <v>23.71529713153314</v>
-      </c>
-      <c r="C34" s="40" t="n">
+      <c r="B34" s="14" t="n">
+        <v>23.71354116704756</v>
+      </c>
+      <c r="C34" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="D34" s="40" t="n">
-        <v>23.71529713153314</v>
-      </c>
-      <c r="E34" s="46" t="n">
-        <v>-1.284702868466862</v>
-      </c>
-      <c r="F34" s="47" t="inlineStr">
+      <c r="D34" s="14" t="n">
+        <v>23.71354116704756</v>
+      </c>
+      <c r="E34" s="44" t="n">
+        <v>-1.286458832952437</v>
+      </c>
+      <c r="F34" s="45" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1771,19 +1763,19 @@
           <t>CSPX.L</t>
         </is>
       </c>
-      <c r="B35" s="43" t="n">
-        <v>19.04164641687945</v>
-      </c>
-      <c r="C35" s="43" t="n">
+      <c r="B35" s="18" t="n">
+        <v>19.04223790988896</v>
+      </c>
+      <c r="C35" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="D35" s="43" t="n">
-        <v>19.04164641687945</v>
-      </c>
-      <c r="E35" s="48" t="n">
-        <v>-0.9583535831205516</v>
-      </c>
-      <c r="F35" s="49" t="inlineStr">
+      <c r="D35" s="18" t="n">
+        <v>19.04223790988896</v>
+      </c>
+      <c r="E35" s="46" t="n">
+        <v>-0.9577620901110357</v>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
         <is>
           <t>● Aligned</t>
         </is>
@@ -1834,19 +1826,19 @@
           <t>IBTM.L</t>
         </is>
       </c>
-      <c r="B39" s="40" t="n">
+      <c r="B39" s="14" t="n">
         <v>35.68082636471589</v>
       </c>
-      <c r="C39" s="40" t="n">
+      <c r="C39" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="D39" s="40" t="n">
+      <c r="D39" s="14" t="n">
         <v>35.68082636471589</v>
       </c>
-      <c r="E39" s="50" t="n">
+      <c r="E39" s="48" t="n">
         <v>5.680826364715891</v>
       </c>
-      <c r="F39" s="51" t="inlineStr">
+      <c r="F39" s="49" t="inlineStr">
         <is>
           <t>● Action</t>
         </is>
@@ -1858,19 +1850,19 @@
           <t>IEAG.L</t>
         </is>
       </c>
-      <c r="B40" s="43" t="n">
+      <c r="B40" s="18" t="n">
         <v>64.31917363528412</v>
       </c>
-      <c r="C40" s="43" t="n">
+      <c r="C40" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="D40" s="43" t="n">
+      <c r="D40" s="18" t="n">
         <v>64.31917363528412</v>
       </c>
-      <c r="E40" s="52" t="n">
+      <c r="E40" s="50" t="n">
         <v>-5.680826364715884</v>
       </c>
-      <c r="F40" s="53" t="inlineStr">
+      <c r="F40" s="51" t="inlineStr">
         <is>
           <t>● Action</t>
         </is>
@@ -1907,7 +1899,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="54" t="inlineStr">
+      <c r="A46" s="52" t="inlineStr">
         <is>
           <t>Alert threshold</t>
         </is>
@@ -1924,7 +1916,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="55" t="inlineStr">
+      <c r="A47" s="53" t="inlineStr">
         <is>
           <t>Solver tolerance</t>
         </is>
@@ -1941,7 +1933,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="54" t="inlineStr">
+      <c r="A48" s="52" t="inlineStr">
         <is>
           <t>Max tolerance</t>
         </is>
@@ -1958,7 +1950,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="55" t="inlineStr">
+      <c r="A49" s="53" t="inlineStr">
         <is>
           <t>Min transaction</t>
         </is>
@@ -1975,7 +1967,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="54" t="inlineStr">
+      <c r="A50" s="52" t="inlineStr">
         <is>
           <t>Lump sum</t>
         </is>
@@ -1992,7 +1984,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="55" t="inlineStr">
+      <c r="A51" s="53" t="inlineStr">
         <is>
           <t>No-sell mode</t>
         </is>
@@ -2011,7 +2003,7 @@
     <row r="53">
       <c r="A53" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:28 v2.0</t>
+          <t>Generated 2026-05-04 13:36 v2.0</t>
         </is>
       </c>
     </row>
@@ -2204,25 +2196,25 @@
         <v>128</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>155.0800018310547</v>
+        <v>155.1000061035156</v>
       </c>
       <c r="J4" s="28" t="n">
         <v>10240</v>
       </c>
       <c r="K4" s="28" t="n">
-        <v>12406.40014648438</v>
+        <v>12408.00048828125</v>
       </c>
       <c r="L4" s="29" t="n">
-        <v>15.35051232088437</v>
+        <v>15.35047488934462</v>
       </c>
       <c r="M4" s="29" t="n">
-        <v>23.71529713153314</v>
+        <v>23.71354116704756</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>2166.400146484375</v>
+        <v>2168.00048828125</v>
       </c>
       <c r="O4" s="29" t="n">
-        <v>21.15625143051147</v>
+        <v>21.17187976837158</v>
       </c>
       <c r="P4" s="27" t="inlineStr">
         <is>
@@ -2241,7 +2233,7 @@
       </c>
       <c r="S4" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2292,10 +2284,10 @@
         <v>11547.61339873075</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>14.2879303956883</v>
+        <v>14.28605275092394</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>22.07369419634397</v>
+        <v>22.06921300257647</v>
       </c>
       <c r="N5" s="32" t="n">
         <v>9307.613398730755</v>
@@ -2320,7 +2312,7 @@
       </c>
       <c r="S5" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2362,25 +2354,25 @@
         <v>570</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>664.0953687273905</v>
+        <v>664.2508475627146</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>8550</v>
       </c>
       <c r="K6" s="28" t="n">
-        <v>9961.430530910857</v>
+        <v>9963.762713440719</v>
       </c>
       <c r="L6" s="29" t="n">
-        <v>12.32533694648823</v>
+        <v>12.32660245947866</v>
       </c>
       <c r="M6" s="29" t="n">
-        <v>19.04164641687945</v>
+        <v>19.04223790988896</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>1411.430530910857</v>
+        <v>1413.762713440719</v>
       </c>
       <c r="O6" s="29" t="n">
-        <v>16.50795942585797</v>
+        <v>16.53523641451134</v>
       </c>
       <c r="P6" s="27" t="inlineStr">
         <is>
@@ -2399,7 +2391,7 @@
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2441,25 +2433,25 @@
         <v>56</v>
       </c>
       <c r="I7" s="32" t="n">
-        <v>76.16799926757812</v>
+        <v>76.19400024414062</v>
       </c>
       <c r="J7" s="32" t="n">
         <v>5040</v>
       </c>
       <c r="K7" s="32" t="n">
-        <v>6855.119934082031</v>
+        <v>6857.460021972656</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>8.481880462245561</v>
+        <v>8.483660842163392</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>13.10381772226808</v>
+        <v>13.10562976573164</v>
       </c>
       <c r="N7" s="32" t="n">
-        <v>1815.119934082031</v>
+        <v>1817.460021972656</v>
       </c>
       <c r="O7" s="33" t="n">
-        <v>36.01428440638951</v>
+        <v>36.06071472167969</v>
       </c>
       <c r="P7" s="31" t="inlineStr">
         <is>
@@ -2478,7 +2470,7 @@
       </c>
       <c r="S7" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2520,25 +2512,25 @@
         <v>98</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>117.754997253418</v>
+        <v>117.7699966430664</v>
       </c>
       <c r="J8" s="28" t="n">
         <v>4900</v>
       </c>
       <c r="K8" s="28" t="n">
-        <v>5887.749862670898</v>
+        <v>5888.49983215332</v>
       </c>
       <c r="L8" s="29" t="n">
-        <v>7.284947748104517</v>
+        <v>7.284918218269714</v>
       </c>
       <c r="M8" s="29" t="n">
-        <v>11.25465370943649</v>
+        <v>11.25380219913764</v>
       </c>
       <c r="N8" s="28" t="n">
-        <v>987.7498626708984</v>
+        <v>988.4998321533203</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>20.1581604626714</v>
+        <v>20.17346596231266</v>
       </c>
       <c r="P8" s="27" t="inlineStr">
         <is>
@@ -2557,7 +2549,7 @@
       </c>
       <c r="S8" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2599,25 +2591,25 @@
         <v>33</v>
       </c>
       <c r="I9" s="32" t="n">
-        <v>47.13000106811523</v>
+        <v>47.15999984741211</v>
       </c>
       <c r="J9" s="32" t="n">
         <v>3960</v>
       </c>
       <c r="K9" s="32" t="n">
-        <v>5655.600128173828</v>
+        <v>5659.199981689453</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v>6.997707507776049</v>
+        <v>7.001241440532606</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v>10.81089082353887</v>
+        <v>10.81557595561772</v>
       </c>
       <c r="N9" s="32" t="n">
-        <v>1695.600128173828</v>
+        <v>1699.199981689453</v>
       </c>
       <c r="O9" s="33" t="n">
-        <v>42.81818505489465</v>
+        <v>42.90909044670336</v>
       </c>
       <c r="P9" s="31" t="inlineStr">
         <is>
@@ -2636,7 +2628,7 @@
       </c>
       <c r="S9" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2679,7 @@
         <v>10715.00015258789</v>
       </c>
       <c r="L10" s="29" t="n">
-        <v>13.25773309892698</v>
+        <v>13.25599083728018</v>
       </c>
       <c r="M10" s="29" t="n">
         <v>64.31917363528412</v>
@@ -2715,7 +2707,7 @@
       </c>
       <c r="S10" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2758,7 @@
         <v>5944.107150852142</v>
       </c>
       <c r="L11" s="33" t="n">
-        <v>7.354678954287075</v>
+        <v>7.353712441009809</v>
       </c>
       <c r="M11" s="33" t="n">
         <v>35.68082636471589</v>
@@ -2794,7 +2786,7 @@
       </c>
       <c r="S11" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2837,7 @@
         <v>5000</v>
       </c>
       <c r="L12" s="29" t="n">
-        <v>6.18652958942094</v>
+        <v>6.185716588197428</v>
       </c>
       <c r="M12" s="29" t="n">
         <v>100</v>
@@ -2873,7 +2865,7 @@
       </c>
       <c r="S12" s="27" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2885,7 @@
           <t>IE00B579F325</t>
         </is>
       </c>
-      <c r="D13" s="56" t="inlineStr">
+      <c r="D13" s="54" t="inlineStr">
         <is>
           <t>Commodities</t>
         </is>
@@ -2924,7 +2916,7 @@
         <v>6847.734948739668</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v>8.472742976177967</v>
+        <v>8.471629532799646</v>
       </c>
       <c r="M13" s="33" t="n">
         <v>100</v>
@@ -2952,14 +2944,14 @@
       </c>
       <c r="S13" s="31" t="inlineStr">
         <is>
-          <t>2026-05-04 13:28</t>
+          <t>2026-05-04 13:36</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:28 v2.0</t>
+          <t>Generated 2026-05-04 13:36 v2.0</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3001,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="57" t="inlineStr">
+      <c r="A2" s="55" t="inlineStr">
         <is>
           <t>Period returns (1D–5Y) and risk metrics calculated on available history per instrument (max 5 years). α/β computed vs S&amp;P 500.</t>
         </is>
@@ -3123,71 +3115,71 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="58" t="inlineStr">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>** TOTAL PORTFOLIO **</t>
         </is>
       </c>
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="57" t="inlineStr">
         <is>
           <t>Portfolio</t>
         </is>
       </c>
-      <c r="C5" s="60" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="D5" s="60" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="E5" s="60" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="F5" s="60" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="G5" s="60" t="n">
-        <v>6.58</v>
-      </c>
-      <c r="H5" s="60" t="n">
-        <v>6.99</v>
-      </c>
-      <c r="I5" s="60" t="n">
-        <v>22</v>
-      </c>
-      <c r="J5" s="60" t="n">
-        <v>48.92</v>
-      </c>
-      <c r="K5" s="60" t="n">
-        <v>45.09</v>
-      </c>
-      <c r="L5" s="60" t="n">
+      <c r="C5" s="58" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D5" s="58" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E5" s="58" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="F5" s="58" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G5" s="58" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H5" s="58" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="58" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="J5" s="58" t="n">
+        <v>48.94</v>
+      </c>
+      <c r="K5" s="58" t="n">
+        <v>45.12</v>
+      </c>
+      <c r="L5" s="58" t="n">
         <v>7.92</v>
       </c>
-      <c r="M5" s="60" t="n">
+      <c r="M5" s="58" t="n">
         <v>8.109999999999999</v>
       </c>
-      <c r="N5" s="60" t="n">
+      <c r="N5" s="58" t="n">
         <v>0.48</v>
       </c>
-      <c r="O5" s="60" t="n">
+      <c r="O5" s="58" t="n">
         <v>0.63</v>
       </c>
-      <c r="P5" s="61" t="n">
+      <c r="P5" s="59" t="n">
         <v>-13.91</v>
       </c>
-      <c r="Q5" s="61" t="n">
+      <c r="Q5" s="59" t="n">
         <v>-0.77</v>
       </c>
-      <c r="R5" s="61" t="n">
+      <c r="R5" s="59" t="n">
         <v>-1.22</v>
       </c>
-      <c r="S5" s="60" t="n">
+      <c r="S5" s="58" t="n">
         <v>2.68</v>
       </c>
-      <c r="T5" s="60" t="n">
+      <c r="T5" s="58" t="n">
         <v>0.15</v>
       </c>
-      <c r="U5" s="59" t="inlineStr">
+      <c r="U5" s="57" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
@@ -3243,13 +3235,13 @@
       <c r="O6" s="29" t="n">
         <v>0.73</v>
       </c>
-      <c r="P6" s="62" t="n">
+      <c r="P6" s="60" t="n">
         <v>-20.22</v>
       </c>
-      <c r="Q6" s="62" t="n">
+      <c r="Q6" s="60" t="n">
         <v>-1.4</v>
       </c>
-      <c r="R6" s="62" t="n">
+      <c r="R6" s="60" t="n">
         <v>-2.13</v>
       </c>
       <c r="S6" s="29" t="n">
@@ -3276,10 +3268,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>6.64</v>
@@ -3288,19 +3280,19 @@
         <v>4.46</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>6.38</v>
+        <v>6.39</v>
       </c>
       <c r="H7" s="33" t="n">
         <v>6.52</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>23.68</v>
+        <v>23.69</v>
       </c>
       <c r="J7" s="33" t="n">
         <v>56.16</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>58.73</v>
+        <v>58.74</v>
       </c>
       <c r="L7" s="33" t="n">
         <v>9.83</v>
@@ -3314,16 +3306,16 @@
       <c r="O7" s="33" t="n">
         <v>0.55</v>
       </c>
-      <c r="P7" s="63" t="n">
+      <c r="P7" s="61" t="n">
         <v>-20.07</v>
       </c>
-      <c r="Q7" s="63" t="n">
+      <c r="Q7" s="61" t="n">
         <v>-1.44</v>
       </c>
-      <c r="R7" s="63" t="n">
+      <c r="R7" s="61" t="n">
         <v>-2.13</v>
       </c>
-      <c r="S7" s="63" t="n">
+      <c r="S7" s="61" t="n">
         <v>-0.49</v>
       </c>
       <c r="T7" s="33" t="n">
@@ -3346,10 +3338,10 @@
           <t>Benchmark index</t>
         </is>
       </c>
-      <c r="C8" s="62" t="n">
+      <c r="C8" s="60" t="n">
         <v>-0.59</v>
       </c>
-      <c r="D8" s="62" t="n">
+      <c r="D8" s="60" t="n">
         <v>-0.06</v>
       </c>
       <c r="E8" s="29" t="n">
@@ -3385,16 +3377,16 @@
       <c r="O8" s="29" t="n">
         <v>0.44</v>
       </c>
-      <c r="P8" s="62" t="n">
+      <c r="P8" s="60" t="n">
         <v>-17.35</v>
       </c>
-      <c r="Q8" s="62" t="n">
+      <c r="Q8" s="60" t="n">
         <v>-1.63</v>
       </c>
-      <c r="R8" s="62" t="n">
+      <c r="R8" s="60" t="n">
         <v>-2.43</v>
       </c>
-      <c r="S8" s="62" t="n">
+      <c r="S8" s="60" t="n">
         <v>-1.39</v>
       </c>
       <c r="T8" s="29" t="n">
@@ -3417,7 +3409,7 @@
           <t>Benchmark index</t>
         </is>
       </c>
-      <c r="C9" s="63" t="n">
+      <c r="C9" s="61" t="n">
         <v>-0.16</v>
       </c>
       <c r="D9" s="33" t="n">
@@ -3456,16 +3448,16 @@
       <c r="O9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="P9" s="63" t="n">
+      <c r="P9" s="61" t="n">
         <v>-24.81</v>
       </c>
-      <c r="Q9" s="63" t="n">
+      <c r="Q9" s="61" t="n">
         <v>-1.93</v>
       </c>
-      <c r="R9" s="63" t="n">
+      <c r="R9" s="61" t="n">
         <v>-2.72</v>
       </c>
-      <c r="S9" s="63" t="n">
+      <c r="S9" s="61" t="n">
         <v>-3.89</v>
       </c>
       <c r="T9" s="33" t="n">
@@ -3495,7 +3487,7 @@
         <v>0.59</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>5.96</v>
+        <v>5.97</v>
       </c>
       <c r="F10" s="29" t="n">
         <v>3.97</v>
@@ -3513,7 +3505,7 @@
         <v>55.69</v>
       </c>
       <c r="K10" s="29" t="n">
-        <v>63.29</v>
+        <v>63.3</v>
       </c>
       <c r="L10" s="29" t="n">
         <v>10.47</v>
@@ -3527,16 +3519,16 @@
       <c r="O10" s="29" t="n">
         <v>0.52</v>
       </c>
-      <c r="P10" s="62" t="n">
+      <c r="P10" s="60" t="n">
         <v>-20.63</v>
       </c>
-      <c r="Q10" s="62" t="n">
+      <c r="Q10" s="60" t="n">
         <v>-1.56</v>
       </c>
-      <c r="R10" s="62" t="n">
+      <c r="R10" s="60" t="n">
         <v>-2.29</v>
       </c>
-      <c r="S10" s="62" t="n">
+      <c r="S10" s="60" t="n">
         <v>-0.5600000000000001</v>
       </c>
       <c r="T10" s="29" t="n">
@@ -3598,13 +3590,13 @@
       <c r="O11" s="33" t="n">
         <v>0.55</v>
       </c>
-      <c r="P11" s="63" t="n">
+      <c r="P11" s="61" t="n">
         <v>-25.91</v>
       </c>
-      <c r="Q11" s="63" t="n">
+      <c r="Q11" s="61" t="n">
         <v>-2.26</v>
       </c>
-      <c r="R11" s="63" t="n">
+      <c r="R11" s="61" t="n">
         <v>-3.15</v>
       </c>
       <c r="S11" s="33" t="n">
@@ -3630,10 +3622,10 @@
           <t>Benchmark index</t>
         </is>
       </c>
-      <c r="C12" s="62" t="n">
+      <c r="C12" s="60" t="n">
         <v>-0.42</v>
       </c>
-      <c r="D12" s="62" t="n">
+      <c r="D12" s="60" t="n">
         <v>-0.5</v>
       </c>
       <c r="E12" s="29" t="n">
@@ -3669,16 +3661,16 @@
       <c r="O12" s="29" t="n">
         <v>0.61</v>
       </c>
-      <c r="P12" s="62" t="n">
+      <c r="P12" s="60" t="n">
         <v>-22.45</v>
       </c>
-      <c r="Q12" s="62" t="n">
+      <c r="Q12" s="60" t="n">
         <v>-1.79</v>
       </c>
-      <c r="R12" s="62" t="n">
+      <c r="R12" s="60" t="n">
         <v>-2.66</v>
       </c>
-      <c r="S12" s="62" t="n">
+      <c r="S12" s="60" t="n">
         <v>-0.13</v>
       </c>
       <c r="T12" s="29" t="n">
@@ -3740,13 +3732,13 @@
       <c r="O13" s="33" t="n">
         <v>0.7</v>
       </c>
-      <c r="P13" s="63" t="n">
+      <c r="P13" s="61" t="n">
         <v>-31.38</v>
       </c>
-      <c r="Q13" s="63" t="n">
+      <c r="Q13" s="61" t="n">
         <v>-2.45</v>
       </c>
-      <c r="R13" s="63" t="n">
+      <c r="R13" s="61" t="n">
         <v>-3.4</v>
       </c>
       <c r="S13" s="33" t="n">
@@ -3772,7 +3764,7 @@
           <t>Benchmark index</t>
         </is>
       </c>
-      <c r="C14" s="62" t="n">
+      <c r="C14" s="60" t="n">
         <v>-0.09</v>
       </c>
       <c r="D14" s="29" t="n">
@@ -3811,13 +3803,13 @@
       <c r="O14" s="29" t="n">
         <v>0.62</v>
       </c>
-      <c r="P14" s="62" t="n">
+      <c r="P14" s="60" t="n">
         <v>-23.17</v>
       </c>
-      <c r="Q14" s="62" t="n">
+      <c r="Q14" s="60" t="n">
         <v>-1.87</v>
       </c>
-      <c r="R14" s="62" t="n">
+      <c r="R14" s="60" t="n">
         <v>-2.64</v>
       </c>
       <c r="S14" s="29" t="n">
@@ -3846,16 +3838,16 @@
       <c r="C15" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="63" t="n">
+      <c r="D15" s="61" t="n">
         <v>-0.11</v>
       </c>
       <c r="E15" s="33" t="n">
         <v>0.38</v>
       </c>
-      <c r="F15" s="63" t="n">
+      <c r="F15" s="61" t="n">
         <v>-0.8</v>
       </c>
-      <c r="G15" s="63" t="n">
+      <c r="G15" s="61" t="n">
         <v>-0.64</v>
       </c>
       <c r="H15" s="33" t="n">
@@ -3867,31 +3859,31 @@
       <c r="J15" s="33" t="n">
         <v>7.86</v>
       </c>
-      <c r="K15" s="63" t="n">
+      <c r="K15" s="61" t="n">
         <v>-8.98</v>
       </c>
-      <c r="L15" s="63" t="n">
+      <c r="L15" s="61" t="n">
         <v>-1.87</v>
       </c>
       <c r="M15" s="33" t="n">
         <v>5.55</v>
       </c>
-      <c r="N15" s="63" t="n">
+      <c r="N15" s="61" t="n">
         <v>-1.06</v>
       </c>
-      <c r="O15" s="63" t="n">
+      <c r="O15" s="61" t="n">
         <v>-1.63</v>
       </c>
-      <c r="P15" s="63" t="n">
+      <c r="P15" s="61" t="n">
         <v>-19.81</v>
       </c>
-      <c r="Q15" s="63" t="n">
+      <c r="Q15" s="61" t="n">
         <v>-0.55</v>
       </c>
-      <c r="R15" s="63" t="n">
+      <c r="R15" s="61" t="n">
         <v>-0.77</v>
       </c>
-      <c r="S15" s="63" t="n">
+      <c r="S15" s="61" t="n">
         <v>-6</v>
       </c>
       <c r="T15" s="33" t="n">
@@ -3915,34 +3907,34 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>7.75</v>
+        <v>7.77</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>4.71</v>
+        <v>4.73</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>6.61</v>
+        <v>6.63</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>6.85</v>
+        <v>6.86</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>24.62</v>
+        <v>24.64</v>
       </c>
       <c r="J16" s="29" t="n">
-        <v>62.81</v>
+        <v>62.83</v>
       </c>
       <c r="K16" s="29" t="n">
-        <v>70.29000000000001</v>
+        <v>70.31</v>
       </c>
       <c r="L16" s="29" t="n">
-        <v>11.52</v>
+        <v>11.53</v>
       </c>
       <c r="M16" s="29" t="n">
         <v>13.8</v>
@@ -3953,13 +3945,13 @@
       <c r="O16" s="29" t="n">
         <v>0.7</v>
       </c>
-      <c r="P16" s="62" t="n">
+      <c r="P16" s="60" t="n">
         <v>-21.07</v>
       </c>
-      <c r="Q16" s="62" t="n">
+      <c r="Q16" s="60" t="n">
         <v>-1.39</v>
       </c>
-      <c r="R16" s="62" t="n">
+      <c r="R16" s="60" t="n">
         <v>-2.13</v>
       </c>
       <c r="S16" s="29" t="n">
@@ -3977,7 +3969,7 @@
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
         </is>
       </c>
       <c r="B17" s="31" t="inlineStr">
@@ -3986,58 +3978,58 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>0.62</v>
+        <v>1.87</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>0.96</v>
+        <v>1.45</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>7.32</v>
+        <v>12.64</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>4.24</v>
+        <v>8.94</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>5.39</v>
+        <v>16.56</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>5.78</v>
+        <v>16.16</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>22.94</v>
+        <v>40.77</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>62.65</v>
+        <v>68.70999999999999</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>75.11</v>
+        <v>42.17</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v>12.16</v>
+        <v>7.57</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>14.24</v>
+        <v>18.83</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>0.57</v>
+        <v>0.19</v>
       </c>
       <c r="O17" s="33" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="P17" s="63" t="n">
-        <v>-21.73</v>
-      </c>
-      <c r="Q17" s="63" t="n">
-        <v>-1.45</v>
-      </c>
-      <c r="R17" s="63" t="n">
-        <v>-2.19</v>
+        <v>0.26</v>
+      </c>
+      <c r="P17" s="61" t="n">
+        <v>-24.38</v>
+      </c>
+      <c r="Q17" s="61" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="R17" s="61" t="n">
+        <v>-2.59</v>
       </c>
       <c r="S17" s="33" t="n">
-        <v>6.35</v>
+        <v>2.75</v>
       </c>
       <c r="T17" s="33" t="n">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="U17" s="31" t="inlineStr">
         <is>
@@ -4048,7 +4040,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI Emerging Markets UCITS ETF 1C</t>
+          <t>iShares VII PLC - iShares Core S&amp;P 500 UCITS ETF</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -4056,59 +4048,59 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C18" s="29" t="n">
-        <v>1.83</v>
+      <c r="C18" s="60" t="n">
+        <v>-0.09</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>1.42</v>
+        <v>1.16</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>12.6</v>
+        <v>8.83</v>
       </c>
       <c r="F18" s="29" t="n">
-        <v>8.9</v>
+        <v>5.43</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>16.52</v>
+        <v>4.81</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>16.12</v>
+        <v>6.41</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>40.72</v>
+        <v>25.3</v>
       </c>
       <c r="J18" s="29" t="n">
-        <v>68.66</v>
+        <v>70.91</v>
       </c>
       <c r="K18" s="29" t="n">
-        <v>42.12</v>
+        <v>88.41</v>
       </c>
       <c r="L18" s="29" t="n">
-        <v>7.56</v>
+        <v>13.83</v>
       </c>
       <c r="M18" s="29" t="n">
-        <v>18.82</v>
+        <v>17.29</v>
       </c>
       <c r="N18" s="29" t="n">
-        <v>0.19</v>
+        <v>0.57</v>
       </c>
       <c r="O18" s="29" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="P18" s="62" t="n">
-        <v>-24.38</v>
-      </c>
-      <c r="Q18" s="62" t="n">
-        <v>-1.59</v>
-      </c>
-      <c r="R18" s="62" t="n">
-        <v>-2.59</v>
+        <v>0.79</v>
+      </c>
+      <c r="P18" s="60" t="n">
+        <v>-22.73</v>
+      </c>
+      <c r="Q18" s="60" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="R18" s="60" t="n">
+        <v>-2.53</v>
       </c>
       <c r="S18" s="29" t="n">
-        <v>2.74</v>
+        <v>6.37</v>
       </c>
       <c r="T18" s="29" t="n">
-        <v>0.1</v>
+        <v>0.42</v>
       </c>
       <c r="U18" s="27" t="inlineStr">
         <is>
@@ -4119,7 +4111,7 @@
     <row r="19">
       <c r="A19" s="31" t="inlineStr">
         <is>
-          <t>iShares VII PLC - iShares Core S&amp;P 500 UCITS ETF</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="B19" s="31" t="inlineStr">
@@ -4127,59 +4119,59 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C19" s="63" t="n">
-        <v>-0.11</v>
+      <c r="C19" s="33" t="n">
+        <v>0.63</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>1.13</v>
+        <v>0.98</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>8.81</v>
+        <v>7.33</v>
       </c>
       <c r="F19" s="33" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G19" s="33" t="n">
         <v>5.4</v>
       </c>
-      <c r="G19" s="33" t="n">
-        <v>4.78</v>
-      </c>
       <c r="H19" s="33" t="n">
-        <v>6.38</v>
+        <v>5.79</v>
       </c>
       <c r="I19" s="33" t="n">
-        <v>25.28</v>
+        <v>22.96</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>70.87</v>
+        <v>62.67</v>
       </c>
       <c r="K19" s="33" t="n">
-        <v>88.36</v>
+        <v>75.13</v>
       </c>
       <c r="L19" s="33" t="n">
-        <v>13.82</v>
+        <v>12.17</v>
       </c>
       <c r="M19" s="33" t="n">
-        <v>17.29</v>
+        <v>14.24</v>
       </c>
       <c r="N19" s="33" t="n">
         <v>0.57</v>
       </c>
       <c r="O19" s="33" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="P19" s="63" t="n">
-        <v>-22.73</v>
-      </c>
-      <c r="Q19" s="63" t="n">
-        <v>-1.73</v>
-      </c>
-      <c r="R19" s="63" t="n">
-        <v>-2.53</v>
+        <v>0.73</v>
+      </c>
+      <c r="P19" s="61" t="n">
+        <v>-21.73</v>
+      </c>
+      <c r="Q19" s="61" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="R19" s="61" t="n">
+        <v>-2.19</v>
       </c>
       <c r="S19" s="33" t="n">
         <v>6.36</v>
       </c>
       <c r="T19" s="33" t="n">
-        <v>0.42</v>
+        <v>0.22</v>
       </c>
       <c r="U19" s="31" t="inlineStr">
         <is>
@@ -4201,55 +4193,55 @@
       <c r="C20" s="29" t="n">
         <v>0.31</v>
       </c>
-      <c r="D20" s="62" t="n">
+      <c r="D20" s="60" t="n">
         <v>-0.7</v>
       </c>
-      <c r="E20" s="62" t="n">
+      <c r="E20" s="60" t="n">
         <v>-1.11</v>
       </c>
       <c r="F20" s="29" t="n">
         <v>0.9</v>
       </c>
-      <c r="G20" s="62" t="n">
+      <c r="G20" s="60" t="n">
         <v>-1.55</v>
       </c>
       <c r="H20" s="29" t="n">
         <v>0.02</v>
       </c>
-      <c r="I20" s="62" t="n">
+      <c r="I20" s="60" t="n">
         <v>-0.52</v>
       </c>
-      <c r="J20" s="62" t="n">
+      <c r="J20" s="60" t="n">
         <v>-0.82</v>
       </c>
-      <c r="K20" s="62" t="n">
+      <c r="K20" s="60" t="n">
         <v>-1.61</v>
       </c>
-      <c r="L20" s="62" t="n">
+      <c r="L20" s="60" t="n">
         <v>-0.33</v>
       </c>
       <c r="M20" s="29" t="n">
         <v>10.65</v>
       </c>
-      <c r="N20" s="62" t="n">
+      <c r="N20" s="60" t="n">
         <v>-0.41</v>
       </c>
-      <c r="O20" s="62" t="n">
+      <c r="O20" s="60" t="n">
         <v>-0.61</v>
       </c>
-      <c r="P20" s="62" t="n">
+      <c r="P20" s="60" t="n">
         <v>-15.77</v>
       </c>
-      <c r="Q20" s="62" t="n">
+      <c r="Q20" s="60" t="n">
         <v>-1.1</v>
       </c>
-      <c r="R20" s="62" t="n">
+      <c r="R20" s="60" t="n">
         <v>-1.48</v>
       </c>
-      <c r="S20" s="62" t="n">
+      <c r="S20" s="60" t="n">
         <v>-4.14</v>
       </c>
-      <c r="T20" s="62" t="n">
+      <c r="T20" s="60" t="n">
         <v>-0.02</v>
       </c>
       <c r="U20" s="27" t="inlineStr">
@@ -4269,13 +4261,13 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C21" s="63" t="n">
+      <c r="C21" s="61" t="n">
         <v>-0.1</v>
       </c>
-      <c r="D21" s="63" t="n">
+      <c r="D21" s="61" t="n">
         <v>-2.09</v>
       </c>
-      <c r="E21" s="63" t="n">
+      <c r="E21" s="61" t="n">
         <v>-4.21</v>
       </c>
       <c r="F21" s="33" t="n">
@@ -4308,13 +4300,13 @@
       <c r="O21" s="33" t="n">
         <v>1.36</v>
       </c>
-      <c r="P21" s="63" t="n">
+      <c r="P21" s="61" t="n">
         <v>-15.94</v>
       </c>
-      <c r="Q21" s="63" t="n">
+      <c r="Q21" s="61" t="n">
         <v>-1.75</v>
       </c>
-      <c r="R21" s="63" t="n">
+      <c r="R21" s="61" t="n">
         <v>-2.57</v>
       </c>
       <c r="S21" s="33" t="n">
@@ -4379,13 +4371,13 @@
       <c r="O22" s="29" t="n">
         <v>0.46</v>
       </c>
-      <c r="P22" s="62" t="n">
+      <c r="P22" s="60" t="n">
         <v>-21.24</v>
       </c>
-      <c r="Q22" s="62" t="n">
+      <c r="Q22" s="60" t="n">
         <v>-1.78</v>
       </c>
-      <c r="R22" s="62" t="n">
+      <c r="R22" s="60" t="n">
         <v>-2.5</v>
       </c>
       <c r="S22" s="29" t="n">
@@ -4411,56 +4403,56 @@
           <t>In portfolio</t>
         </is>
       </c>
-      <c r="C23" s="63" t="n">
-        <v>-0.5600000000000001</v>
-      </c>
-      <c r="D23" s="63" t="n">
-        <v>-0.11</v>
+      <c r="C23" s="61" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="D23" s="61" t="n">
+        <v>-0.04</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>4.09</v>
-      </c>
-      <c r="F23" s="63" t="n">
-        <v>-1.19</v>
+        <v>4.15</v>
+      </c>
+      <c r="F23" s="61" t="n">
+        <v>-1.13</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>6.97</v>
+        <v>7.03</v>
       </c>
       <c r="H23" s="33" t="n">
-        <v>2.04</v>
+        <v>2.11</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>14.28</v>
+        <v>14.35</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>40.02</v>
+        <v>40.11</v>
       </c>
       <c r="K23" s="33" t="n">
-        <v>54.34</v>
+        <v>54.43</v>
       </c>
       <c r="L23" s="33" t="n">
-        <v>9.48</v>
+        <v>9.49</v>
       </c>
       <c r="M23" s="33" t="n">
-        <v>14.95</v>
+        <v>14.94</v>
       </c>
       <c r="N23" s="33" t="n">
         <v>0.37</v>
       </c>
       <c r="O23" s="33" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="P23" s="63" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P23" s="61" t="n">
         <v>-22.86</v>
       </c>
-      <c r="Q23" s="63" t="n">
+      <c r="Q23" s="61" t="n">
         <v>-1.53</v>
       </c>
-      <c r="R23" s="63" t="n">
+      <c r="R23" s="61" t="n">
         <v>-2.22</v>
       </c>
       <c r="S23" s="33" t="n">
-        <v>4.06</v>
+        <v>4.07</v>
       </c>
       <c r="T23" s="33" t="n">
         <v>0.17</v>
@@ -4472,7 +4464,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="64" t="inlineStr">
+      <c r="A26" s="62" t="inlineStr">
         <is>
           <t>Legend — Rating Thresholds</t>
         </is>
@@ -4516,7 +4508,7 @@
           <t>CAGR</t>
         </is>
       </c>
-      <c r="B28" s="65" t="inlineStr">
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>Compound Annual Growth Rate. The single yearly return that, if repeated every year, would grow your portfolio from start to end value. Accounts for compounding. ~7% is the long-term global equity average.</t>
         </is>
@@ -4548,7 +4540,7 @@
           <t>α (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="B29" s="66" t="inlineStr">
+      <c r="B29" s="64" t="inlineStr">
         <is>
           <t>Extra annual return vs the benchmark, after adjusting for how risky the portfolio is (CAPM). Positive = you beat the market beyond what your risk alone justified. Negative = you underperformed after fees and noise.</t>
         </is>
@@ -4580,7 +4572,7 @@
           <t>β (vs S&amp;P 500)</t>
         </is>
       </c>
-      <c r="B30" s="65" t="inlineStr">
+      <c r="B30" s="63" t="inlineStr">
         <is>
           <t>How much your portfolio moves when the benchmark moves 1%. β=1 in line, β=0.5 half as reactive, β=1.5 amplifies by 50%, β≈0 uncorrelated. Tells you how much systematic market risk you're running.</t>
         </is>
@@ -4612,7 +4604,7 @@
           <t>Max DD</t>
         </is>
       </c>
-      <c r="B31" s="66" t="inlineStr">
+      <c r="B31" s="64" t="inlineStr">
         <is>
           <t>Maximum Drawdown. Worst peak-to-trough loss over the period — the most painful scenario an investor lived through. -20% is typical for diversified equity; deeper drops signal concentration or high volatility.</t>
         </is>
@@ -4644,7 +4636,7 @@
           <t>Volatility</t>
         </is>
       </c>
-      <c r="B32" s="65" t="inlineStr">
+      <c r="B32" s="63" t="inlineStr">
         <is>
           <t>How bumpy the ride is. Annualized standard deviation of daily returns. A 15% vol means ~±15% year-to-year noise around the average return. Equity indexes ~15–20%, bonds ~3–7%.</t>
         </is>
@@ -4676,7 +4668,7 @@
           <t>Sharpe</t>
         </is>
       </c>
-      <c r="B33" s="66" t="inlineStr">
+      <c r="B33" s="64" t="inlineStr">
         <is>
           <t>Return per unit of risk taken: (CAGR − risk-free rate) / Volatility. Above 1 is good, above 2 is excellent, negative means you were paid less than a safe bond for the risk you ran.</t>
         </is>
@@ -4708,7 +4700,7 @@
           <t>Sortino</t>
         </is>
       </c>
-      <c r="B34" s="65" t="inlineStr">
+      <c r="B34" s="63" t="inlineStr">
         <is>
           <t>Like Sharpe but only penalizes downside volatility (ignores upside swings). More honest when returns are asymmetric. Usually higher than Sharpe — the gap shows how much of your volatility is actually good volatility.</t>
         </is>
@@ -4740,7 +4732,7 @@
           <t>VaR 95%</t>
         </is>
       </c>
-      <c r="B35" s="66" t="inlineStr">
+      <c r="B35" s="64" t="inlineStr">
         <is>
           <t>Value at Risk. The daily loss exceeded only 5% of the time (historical simulation). A VaR of -1.2% means on an average month you should expect about one day worse than -1.2%. Non-parametric: no normal-distribution assumption.</t>
         </is>
@@ -4772,7 +4764,7 @@
           <t>CVaR 95%</t>
         </is>
       </c>
-      <c r="B36" s="65" t="inlineStr">
+      <c r="B36" s="63" t="inlineStr">
         <is>
           <t>Conditional VaR, a.k.a. Expected Shortfall. The average loss on the worst 5% of days. Always more negative than VaR. Captures tail risk VaR misses — how bad it really gets when it goes bad.</t>
         </is>
@@ -4801,7 +4793,7 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>Generated 2026-05-04 13:28 v2.0</t>
+          <t>Generated 2026-05-04 13:36 v2.0</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4833,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="64" t="inlineStr">
+      <c r="A3" s="62" t="inlineStr">
         <is>
           <t>Return Contribution by Holding</t>
         </is>
@@ -4896,13 +4888,13 @@
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>14.2879303956883</v>
+        <v>14.28605275092394</v>
       </c>
       <c r="E5" s="29" t="n">
         <v>415.5184553004801</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>59.36898767457182</v>
+        <v>59.3611857140509</v>
       </c>
     </row>
     <row r="6">
@@ -4922,13 +4914,13 @@
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>13.25773309892698</v>
+        <v>13.25599083728018</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>91.33928843906948</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>12.10951907571089</v>
+        <v>12.10792770631996</v>
       </c>
     </row>
     <row r="7">
@@ -4948,13 +4940,13 @@
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>8.472742976177967</v>
+        <v>8.471629532799646</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>55.27743647935755</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>4.683515116716004</v>
+        <v>4.68289963375982</v>
       </c>
     </row>
     <row r="8">
@@ -4974,13 +4966,13 @@
         </is>
       </c>
       <c r="D8" s="33" t="n">
-        <v>15.35051232088437</v>
+        <v>15.35047488934462</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>21.15625143051147</v>
+        <v>21.17187976837158</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>3.24759298247794</v>
+        <v>3.249984087446114</v>
       </c>
     </row>
     <row r="9">
@@ -5000,13 +4992,13 @@
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>8.481880462245561</v>
+        <v>8.483660842163392</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>36.01428440638951</v>
+        <v>36.06071472167969</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>3.054688552683102</v>
+        <v>3.059268734247389</v>
       </c>
     </row>
     <row r="10">
@@ -5026,13 +5018,13 @@
         </is>
       </c>
       <c r="D10" s="33" t="n">
-        <v>7.354678954287075</v>
+        <v>7.353712441009809</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>41.5263607345748</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>3.054130513427105</v>
+        <v>3.053729155637039</v>
       </c>
     </row>
     <row r="11">
@@ -5052,13 +5044,13 @@
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>6.997707507776049</v>
+        <v>7.001241440532606</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>42.81818505489465</v>
+        <v>42.90909044670336</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>2.996291350279805</v>
+        <v>3.004169022110213</v>
       </c>
     </row>
     <row r="12">
@@ -5078,13 +5070,13 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>12.32533694648823</v>
+        <v>12.32660245947866</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>16.50795942585797</v>
+        <v>16.53523641451134</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>2.034661622226559</v>
+        <v>2.038232858551765</v>
       </c>
     </row>
     <row r="13">
@@ -5104,13 +5096,13 @@
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>7.284947748104517</v>
+        <v>7.284918218269714</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>20.1581604626714</v>
+        <v>20.17346596231266</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>1.468511456684675</v>
+        <v>1.469620497144954</v>
       </c>
     </row>
     <row r="14">
@@ -5130,7 +5122,7 @@
         </is>
       </c>
       <c r="D14" s="33" t="n">
-        <v>6.18652958942094</v>
+        <v>6.185716588197428</v>
       </c>
       <c r="E14" s="33" t="n">
         <v>0</v>
@@ -5140,7 +5132,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="64" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr">
         <is>
           <t>Breakdown by Asset Class</t>
         </is>
@@ -5175,10 +5167,10 @@
         </is>
       </c>
       <c r="B18" s="28" t="n">
-        <v>52313.91400105275</v>
+        <v>52324.53643626816</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>92.02888268013419</v>
+        <v>92.06147376900979</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>6</v>
@@ -5233,7 +5225,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="64" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>Breakdown by Geography (Equity Only)</t>
         </is>
@@ -5263,23 +5255,23 @@
         </is>
       </c>
       <c r="B25" s="29" t="n">
-        <v>41.79626795598796</v>
+        <v>41.79516167143485</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>19.27412377301361</v>
+        <v>19.29352738173186</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="A26" s="54" t="inlineStr">
         <is>
           <t>Emerging Markets</t>
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>15.50380579197923</v>
+        <v>15.50544013183685</v>
       </c>
       <c r="C26" s="33" t="n">
-        <v>28.58526791845049</v>
+        <v>28.61629724502563</v>
       </c>
     </row>
     <row r="27">
@@ -5289,10 +5281,10 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>9.766116970263369</v>
+        <v>9.768936068831742</v>
       </c>
       <c r="C27" s="29" t="n">
-        <v>28.04419898269251</v>
+        <v>28.0848120591292</v>
       </c>
     </row>
     <row r="28">
@@ -5302,10 +5294,10 @@
         </is>
       </c>
       <c r="B28" s="33" t="n">
-        <v>24.19785747467557</v>
+        <v>24.19321790615446</v>
       </c>
       <c r="C28" s="33" t="n">
-        <v>152.2776223978877</v>
+        <v>152.2879336770548</v>
       </c>
     </row>
     <row r="29">
@@ -5315,10 +5307,10 @@
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>8.735951807093869</v>
+        <v>8.737244221742097</v>
       </c>
       <c r="C29" s="29" t="n">
-        <v>28.04419898269251</v>
+        <v>28.0848120591292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>